<commit_message>
Add the Dorbu dose-response slope to the extraction pipeline
New Vehicle Extraction row: 0.194 g/L of hemoglobin per mg/day of fortificant
iron (95% CrI 0.009-0.446), from Dorbu et al. 2026 (Matern Child Nutr
22:e13801), the same Bayesian meta-regression whose per-vehicle trial-mean
differences we currently apply as fixed shifts. prep_vehicle now splits the
two parameterizations by data point name and emits the slope as
results/iron/fortification_hemoglobin_effect_per_mg.csv; the per-vehicle
mean-difference rows and CSV are retained for reference (verified
byte-identical on rerun).

Groundwork for switching the sims and the 0400 anemia model to a consistent
dose-response iron->hemoglobin relationship (next commits).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpDueU6WT9Sj1m2BsoASHM
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -14868,7 +14868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -15139,6 +15139,49 @@
       <c r="I6" s="6" t="inlineStr">
         <is>
           <t>https://www.bmj.com/content/346/bmj.f3443; study of supplementation at higher doses than fortification; selected the effect among trials &lt;66mg/day as all fortification would fall in this range</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>All (assumed same)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Iron fortification/consumption effect on hemoglobin</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dose-response slope</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>g/L per mg/day</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Dorbu et al. 2026, Matern Child Nutr 22:e13801, doi:10.1111/mcn.13801 (Bayesian meta-regression across 17 fortification trials)</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.009-0.446</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Adopted 2026-08-31, replacing the per-vehicle fixed mean-difference shifts (rows above, retained for reference) so that the hemoglobin effect scales with the delivered iron dose, consistently with the birthweight pathway. Linearity assumed over 0-17 mg/day (trials averaged ~17 mg/day; Luo et al. 2026 make the same assumption). Applied per covered person; the responsive/non-responsive split is handled downstream where applicable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Attempt at the necessary changes to include another scenario (Ethiopia/Salt/Folic acid at 45 ppm)
Not yet tested with a snakemake
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\projects\2026\vivarium_gates_lsff_2026\0100_data_prep\extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6519260-0061-43D4-999E-ACB54C4C2F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39FB672-C793-48C2-A2AD-70ED8B1DFACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Country-Vehicle Progress" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2027" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="236">
   <si>
     <t>Country</t>
   </si>
@@ -760,6 +760,27 @@
   <si>
     <t>J Drive</t>
   </si>
+  <si>
+    <t>Intervention - 45 ppm</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>20260416_Input data to IHME models.xlsx spreadsheet from Jonathan Gorstein, attached to Email 4/16/2026</t>
+  </si>
+  <si>
+    <t>same program reach as the NRV scenarios (Andy Garcia 7/26)</t>
+  </si>
+  <si>
+    <t>45 ppm = 45 µg/g</t>
+  </si>
+  <si>
+    <t>Jonathan Gorstein, 8/15 (same as the 25%/100% NRV scenarios)</t>
+  </si>
+  <si>
+    <t>Kept consistent with the existing NRV scenarios so the three arms differ only in concentration. GF Apr-2026 workbook implies 2030 compliance = 80% (effectiveness 1.0 at 0.8 reach); to be adopted for all Ethiopia scenarios together in the parameter-update batch.</t>
+  </si>
 </sst>
 </file>
 
@@ -769,7 +790,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1367,16 +1388,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="58.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="15.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1395,7 +1416,7 @@
       </c>
       <c r="I1" s="33"/>
     </row>
-    <row r="2" spans="1:9" ht="15">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -1416,7 +1437,7 @@
       </c>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="1:9" ht="15">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -1445,7 +1466,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1456,7 +1477,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:9" ht="15">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1491,7 +1512,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1526,7 +1547,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1561,7 +1582,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1596,7 +1617,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1653,18 +1674,19 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB686F86-0F1B-4E3A-8BF6-0236059233BB}">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="11.42578125" customWidth="1"/>
-    <col min="8" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.453125" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.453125" customWidth="1"/>
+    <col min="9" max="10" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1672,18 +1694,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="33"/>
-      <c r="D1" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33" t="s">
+        <v>2</v>
+      </c>
       <c r="F1" s="33"/>
       <c r="G1" s="33"/>
-      <c r="H1" s="33" t="s">
+      <c r="H1" s="33"/>
+      <c r="I1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="33"/>
-    </row>
-    <row r="2" spans="1:9" ht="15">
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -1691,20 +1714,21 @@
         <v>5</v>
       </c>
       <c r="C2" s="33"/>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="33"/>
+      <c r="E2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33" t="s">
+      <c r="F2" s="33"/>
+      <c r="G2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33" t="s">
+      <c r="H2" s="33"/>
+      <c r="I2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="33"/>
-    </row>
-    <row r="3" spans="1:9" ht="15">
+      <c r="J2" s="33"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>89</v>
       </c>
@@ -1712,26 +1736,27 @@
         <v>90</v>
       </c>
       <c r="C3" s="33"/>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="33"/>
+      <c r="E3" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="F3" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="G3" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="H3" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="I3" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="J3" s="28" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="30" t="s">
         <v>195</v>
       </c>
@@ -1741,8 +1766,8 @@
       <c r="C4" s="31" t="s">
         <v>197</v>
       </c>
-      <c r="D4" s="31" t="s">
-        <v>198</v>
+      <c r="D4" t="s">
+        <v>229</v>
       </c>
       <c r="E4" s="31" t="s">
         <v>198</v>
@@ -1759,139 +1784,151 @@
       <c r="I4" s="31" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="15">
+      <c r="J4" s="31" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="15">
+      <c r="E5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>199</v>
       </c>
       <c r="B6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, B$1,  'Scenario Definition Extraction'!$B$2:$B$997, B$2,  'Scenario Definition Extraction'!$C$2:$C$997, B$3, 'Scenario Definition Extraction'!$D$2:$D$997, B$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="C6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, B$1,  'Scenario Definition Extraction'!$B$2:$B$997, B$2,  'Scenario Definition Extraction'!$C$2:$C$997, B$3, 'Scenario Definition Extraction'!$D$2:$D$997, C$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, C$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="D6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, D$2,  'Scenario Definition Extraction'!$C$2:$C$997, D$3, 'Scenario Definition Extraction'!$D$2:$D$997, D$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+      <c r="D6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E6" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="E6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, D$2,  'Scenario Definition Extraction'!$C$2:$C$997, E$3, 'Scenario Definition Extraction'!$D$2:$D$997, E$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+      <c r="F6" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, F$3, 'Scenario Definition Extraction'!$D$2:$D$1000, F$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="F6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, F$2,  'Scenario Definition Extraction'!$C$2:$C$997, F$3, 'Scenario Definition Extraction'!$D$2:$D$997, F$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+      <c r="G6" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, G$2,  'Scenario Definition Extraction'!$C$2:$C$1000, G$3, 'Scenario Definition Extraction'!$D$2:$D$1000, G$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="G6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, F$2,  'Scenario Definition Extraction'!$C$2:$C$997, G$3, 'Scenario Definition Extraction'!$D$2:$D$997, G$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+      <c r="H6" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, G$2,  'Scenario Definition Extraction'!$C$2:$C$1000, H$3, 'Scenario Definition Extraction'!$D$2:$D$1000, H$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="H6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, H$1,  'Scenario Definition Extraction'!$B$2:$B$997, H$2,  'Scenario Definition Extraction'!$C$2:$C$997, H$3, 'Scenario Definition Extraction'!$D$2:$D$997, H$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+      <c r="I6" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, I$1,  'Scenario Definition Extraction'!$B$2:$B$1000, I$2,  'Scenario Definition Extraction'!$C$2:$C$1000, I$3, 'Scenario Definition Extraction'!$D$2:$D$1000, I$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="I6" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, H$1,  'Scenario Definition Extraction'!$B$2:$B$997, H$2,  'Scenario Definition Extraction'!$C$2:$C$997, I$3, 'Scenario Definition Extraction'!$D$2:$D$997, I$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A6) = 0, "Missing", "Complete")</f>
+      <c r="J6" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, I$1,  'Scenario Definition Extraction'!$B$2:$B$1000, I$2,  'Scenario Definition Extraction'!$C$2:$C$1000, J$3, 'Scenario Definition Extraction'!$D$2:$D$1000, J$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>200</v>
       </c>
       <c r="B7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, B$1,  'Scenario Definition Extraction'!$B$2:$B$997, B$2,  'Scenario Definition Extraction'!$C$2:$C$997, B$3, 'Scenario Definition Extraction'!$D$2:$D$997, B$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="C7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, B$1,  'Scenario Definition Extraction'!$B$2:$B$997, B$2,  'Scenario Definition Extraction'!$C$2:$C$997, B$3, 'Scenario Definition Extraction'!$D$2:$D$997, C$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, C$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="D7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, D$2,  'Scenario Definition Extraction'!$C$2:$C$997, D$3, 'Scenario Definition Extraction'!$D$2:$D$997, D$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+      <c r="D7" t="s">
+        <v>230</v>
+      </c>
+      <c r="E7" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="E7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, D$2,  'Scenario Definition Extraction'!$C$2:$C$997, E$3, 'Scenario Definition Extraction'!$D$2:$D$997, E$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+      <c r="F7" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, F$3, 'Scenario Definition Extraction'!$D$2:$D$1000, F$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="F7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, F$2,  'Scenario Definition Extraction'!$C$2:$C$997, F$3, 'Scenario Definition Extraction'!$D$2:$D$997, F$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+      <c r="G7" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, G$2,  'Scenario Definition Extraction'!$C$2:$C$1000, G$3, 'Scenario Definition Extraction'!$D$2:$D$1000, G$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="G7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, F$2,  'Scenario Definition Extraction'!$C$2:$C$997, G$3, 'Scenario Definition Extraction'!$D$2:$D$997, G$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+      <c r="H7" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, G$2,  'Scenario Definition Extraction'!$C$2:$C$1000, H$3, 'Scenario Definition Extraction'!$D$2:$D$1000, H$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="H7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, H$1,  'Scenario Definition Extraction'!$B$2:$B$997, H$2,  'Scenario Definition Extraction'!$C$2:$C$997, H$3, 'Scenario Definition Extraction'!$D$2:$D$997, H$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+      <c r="I7" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, I$1,  'Scenario Definition Extraction'!$B$2:$B$1000, I$2,  'Scenario Definition Extraction'!$C$2:$C$1000, I$3, 'Scenario Definition Extraction'!$D$2:$D$1000, I$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="I7" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, H$1,  'Scenario Definition Extraction'!$B$2:$B$997, H$2,  'Scenario Definition Extraction'!$C$2:$C$997, I$3, 'Scenario Definition Extraction'!$D$2:$D$997, I$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A7) = 0, "Missing", "Complete")</f>
+      <c r="J7" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, I$1,  'Scenario Definition Extraction'!$B$2:$B$1000, I$2,  'Scenario Definition Extraction'!$C$2:$C$1000, J$3, 'Scenario Definition Extraction'!$D$2:$D$1000, J$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>201</v>
       </c>
       <c r="B8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, B$1,  'Scenario Definition Extraction'!$B$2:$B$997, B$2,  'Scenario Definition Extraction'!$C$2:$C$997, B$3, 'Scenario Definition Extraction'!$D$2:$D$997, B$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="C8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, B$1,  'Scenario Definition Extraction'!$B$2:$B$997, B$2,  'Scenario Definition Extraction'!$C$2:$C$997, B$3, 'Scenario Definition Extraction'!$D$2:$D$997, C$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, C$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="D8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, D$2,  'Scenario Definition Extraction'!$C$2:$C$997, D$3, 'Scenario Definition Extraction'!$D$2:$D$997, D$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+      <c r="D8" t="s">
+        <v>230</v>
+      </c>
+      <c r="E8" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="E8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, D$2,  'Scenario Definition Extraction'!$C$2:$C$997, E$3, 'Scenario Definition Extraction'!$D$2:$D$997, E$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+      <c r="F8" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, F$3, 'Scenario Definition Extraction'!$D$2:$D$1000, F$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="F8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, F$2,  'Scenario Definition Extraction'!$C$2:$C$997, F$3, 'Scenario Definition Extraction'!$D$2:$D$997, F$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+      <c r="G8" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, G$2,  'Scenario Definition Extraction'!$C$2:$C$1000, G$3, 'Scenario Definition Extraction'!$D$2:$D$1000, G$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="G8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, D$1,  'Scenario Definition Extraction'!$B$2:$B$997, F$2,  'Scenario Definition Extraction'!$C$2:$C$997, G$3, 'Scenario Definition Extraction'!$D$2:$D$997, G$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+      <c r="H8" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, G$2,  'Scenario Definition Extraction'!$C$2:$C$1000, H$3, 'Scenario Definition Extraction'!$D$2:$D$1000, H$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="H8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, H$1,  'Scenario Definition Extraction'!$B$2:$B$997, H$2,  'Scenario Definition Extraction'!$C$2:$C$997, H$3, 'Scenario Definition Extraction'!$D$2:$D$997, H$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+      <c r="I8" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, I$1,  'Scenario Definition Extraction'!$B$2:$B$1000, I$2,  'Scenario Definition Extraction'!$C$2:$C$1000, I$3, 'Scenario Definition Extraction'!$D$2:$D$1000, I$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
-      <c r="I8" t="str">
-        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$997, H$1,  'Scenario Definition Extraction'!$B$2:$B$997, H$2,  'Scenario Definition Extraction'!$C$2:$C$997, I$3, 'Scenario Definition Extraction'!$D$2:$D$997, I$4, 'Scenario Definition Extraction'!$E$2:$E$997, $A8) = 0, "Missing", "Complete")</f>
+      <c r="J8" t="str">
+        <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, I$1,  'Scenario Definition Extraction'!$B$2:$B$1000, I$2,  'Scenario Definition Extraction'!$C$2:$C$1000, J$3, 'Scenario Definition Extraction'!$D$2:$D$1000, J$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:I8">
+  <conditionalFormatting sqref="E6:J8 B6:C8">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
@@ -1902,19 +1939,19 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{797B3B46-8F2E-4C67-A115-D7583B1B84DB}">
-  <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.7109375" customWidth="1"/>
-    <col min="5" max="5" width="52.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7265625" customWidth="1"/>
+    <col min="5" max="5" width="52.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="50.42578125" customWidth="1"/>
+    <col min="8" max="8" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="50.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1946,7 +1983,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1975,7 +2012,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2004,7 +2041,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2033,7 +2070,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -2062,7 +2099,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -2094,7 +2131,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -2126,18 +2163,18 @@
         <v>203</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D8" t="s">
-        <v>198</v>
+        <v>229</v>
       </c>
       <c r="E8" t="s">
         <v>200</v>
@@ -2149,16 +2186,16 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
       <c r="I8" s="7">
         <v>0.8</v>
       </c>
       <c r="J8" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2166,7 +2203,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s">
         <v>198</v>
@@ -2190,21 +2227,21 @@
         <v>203</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
         <v>198</v>
       </c>
       <c r="E10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -2213,13 +2250,16 @@
         <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>202</v>
       </c>
       <c r="I10" s="7">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>0.8</v>
+      </c>
+      <c r="J10" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -2227,7 +2267,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D11" t="s">
         <v>198</v>
@@ -2248,15 +2288,15 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
         <v>198</v>
@@ -2271,13 +2311,13 @@
         <v>30</v>
       </c>
       <c r="H12" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I12" s="7">
         <v>0.9</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -2285,7 +2325,7 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D13" t="s">
         <v>198</v>
@@ -2306,18 +2346,18 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C14" t="s">
         <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E14" t="s">
         <v>201</v>
@@ -2329,13 +2369,13 @@
         <v>30</v>
       </c>
       <c r="H14" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I14" s="7">
         <v>0.9</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -2346,7 +2386,7 @@
         <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E15" t="s">
         <v>201</v>
@@ -2364,18 +2404,18 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E16" t="s">
         <v>201</v>
@@ -2387,24 +2427,24 @@
         <v>30</v>
       </c>
       <c r="H16" t="s">
-        <v>202</v>
+        <v>107</v>
       </c>
       <c r="I16" s="7">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
         <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>198</v>
+        <v>229</v>
       </c>
       <c r="E17" t="s">
         <v>201</v>
@@ -2416,18 +2456,21 @@
         <v>30</v>
       </c>
       <c r="H17" t="s">
-        <v>202</v>
+        <v>234</v>
       </c>
       <c r="I17" s="7">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="43.5">
+        <v>0.9</v>
+      </c>
+      <c r="J17" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" t="s">
         <v>91</v>
@@ -2436,30 +2479,27 @@
         <v>198</v>
       </c>
       <c r="E18" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F18" t="s">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="G18" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H18" t="s">
         <v>202</v>
       </c>
-      <c r="I18">
-        <v>1320</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="43.5">
+      <c r="I18" s="7">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" t="s">
         <v>90</v>
@@ -2468,30 +2508,27 @@
         <v>198</v>
       </c>
       <c r="E19" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F19" t="s">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="G19" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H19" t="s">
         <v>202</v>
       </c>
-      <c r="I19">
-        <v>24</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="29.25">
+      <c r="I19" s="7">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" t="s">
         <v>91</v>
@@ -2509,21 +2546,21 @@
         <v>99</v>
       </c>
       <c r="H20" t="s">
-        <v>82</v>
+        <v>202</v>
       </c>
       <c r="I20">
-        <v>40</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="29.25">
+        <v>1320</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C21" t="s">
         <v>90</v>
@@ -2541,27 +2578,27 @@
         <v>99</v>
       </c>
       <c r="H21" t="s">
-        <v>82</v>
+        <v>202</v>
       </c>
       <c r="I21">
-        <v>1.69</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+        <v>24</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D22" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E22" t="s">
         <v>199</v>
@@ -2573,27 +2610,27 @@
         <v>99</v>
       </c>
       <c r="H22" t="s">
-        <v>202</v>
+        <v>82</v>
       </c>
       <c r="I22">
-        <v>14.084507042253522</v>
-      </c>
-      <c r="J22" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>40</v>
+      </c>
+      <c r="J22" s="14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C23" t="s">
         <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E23" t="s">
         <v>199</v>
@@ -2605,27 +2642,27 @@
         <v>99</v>
       </c>
       <c r="H23" t="s">
-        <v>202</v>
+        <v>82</v>
       </c>
       <c r="I23">
-        <v>56.338028169014088</v>
-      </c>
-      <c r="J23" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10">
+        <v>1.69</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E24" t="s">
         <v>199</v>
@@ -2637,27 +2674,27 @@
         <v>99</v>
       </c>
       <c r="H24" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="I24">
-        <v>42.5</v>
+        <v>14.084507042253522</v>
       </c>
       <c r="J24" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="15">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C25" t="s">
         <v>90</v>
       </c>
       <c r="D25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E25" t="s">
         <v>199</v>
@@ -2668,13 +2705,109 @@
       <c r="G25" t="s">
         <v>99</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="H25" t="s">
+        <v>202</v>
+      </c>
+      <c r="I25">
+        <v>56.338028169014088</v>
+      </c>
+      <c r="J25" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" t="s">
+        <v>229</v>
+      </c>
+      <c r="E26" t="s">
+        <v>199</v>
+      </c>
+      <c r="F26" t="s">
+        <v>98</v>
+      </c>
+      <c r="G26" t="s">
+        <v>99</v>
+      </c>
+      <c r="H26" t="s">
+        <v>231</v>
+      </c>
+      <c r="I26">
+        <v>45</v>
+      </c>
+      <c r="J26" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>91</v>
+      </c>
+      <c r="D27" t="s">
+        <v>198</v>
+      </c>
+      <c r="E27" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" t="s">
+        <v>98</v>
+      </c>
+      <c r="G27" t="s">
+        <v>99</v>
+      </c>
+      <c r="H27" t="s">
+        <v>210</v>
+      </c>
+      <c r="I27">
+        <v>42.5</v>
+      </c>
+      <c r="J27" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" t="s">
+        <v>198</v>
+      </c>
+      <c r="E28" t="s">
+        <v>199</v>
+      </c>
+      <c r="F28" t="s">
+        <v>98</v>
+      </c>
+      <c r="G28" t="s">
+        <v>99</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="I25">
+      <c r="I28">
         <v>1.3</v>
       </c>
-      <c r="J25" s="6" t="s">
+      <c r="J28" s="6" t="s">
         <v>213</v>
       </c>
     </row>
@@ -2692,10 +2825,10 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="J25" r:id="rId1" xr:uid="{8B29D165-A493-48F3-B663-85CB453EE758}"/>
-    <hyperlink ref="H25" r:id="rId2" xr:uid="{3DC1B296-F88E-408E-956F-0351AD5F515E}"/>
-    <hyperlink ref="J20" r:id="rId3" xr:uid="{EA845FCE-F931-471E-B7AD-CCDF4F57AEA4}"/>
-    <hyperlink ref="J21" r:id="rId4" xr:uid="{E1E2866D-3A5C-4D33-8B50-C6AA8A296518}"/>
+    <hyperlink ref="J28" r:id="rId1" xr:uid="{8B29D165-A493-48F3-B663-85CB453EE758}"/>
+    <hyperlink ref="H28" r:id="rId2" xr:uid="{3DC1B296-F88E-408E-956F-0351AD5F515E}"/>
+    <hyperlink ref="J22" r:id="rId3" xr:uid="{EA845FCE-F931-471E-B7AD-CCDF4F57AEA4}"/>
+    <hyperlink ref="J23" r:id="rId4" xr:uid="{E1E2866D-3A5C-4D33-8B50-C6AA8A296518}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -2709,7 +2842,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1237FDC8-82EB-4B1F-9280-B2359248B6FE}">
           <x14:formula1>
-            <xm:f>'Scenario Definition Progress'!$B$4:$I$4</xm:f>
+            <xm:f>'Scenario Definition Progress'!$B$4:$J$4</xm:f>
           </x14:formula1>
           <xm:sqref>D1:D1048576</xm:sqref>
         </x14:dataValidation>
@@ -2722,14 +2855,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062B00F0-B806-4CE9-A08D-6C78F3C15B86}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>214</v>
       </c>
@@ -2749,7 +2882,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="43.5">
+    <row r="2" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -2766,7 +2899,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>221</v>
       </c>
@@ -2774,7 +2907,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>223</v>
       </c>
@@ -2806,20 +2939,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7501F0-08E1-4A63-A382-F6741C91E79A}">
   <dimension ref="A1:M106"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="5" max="5" width="60.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.26953125" customWidth="1"/>
+    <col min="5" max="5" width="60.1796875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.140625" customWidth="1"/>
-    <col min="13" max="13" width="50.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="10.1796875" customWidth="1"/>
+    <col min="13" max="13" width="50.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2860,7 +2993,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2892,7 +3025,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2924,7 +3057,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -2953,7 +3086,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -2982,7 +3115,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -3011,7 +3144,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -3040,7 +3173,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -3069,7 +3202,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -3101,7 +3234,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -3130,7 +3263,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -3162,7 +3295,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -3191,7 +3324,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -3220,7 +3353,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -3249,7 +3382,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -3278,7 +3411,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -3307,7 +3440,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -3339,7 +3472,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -3371,7 +3504,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -3409,7 +3542,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -3447,7 +3580,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>2</v>
       </c>
@@ -3485,7 +3618,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -3523,7 +3656,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -3558,7 +3691,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -3593,7 +3726,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -3634,7 +3767,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -3675,7 +3808,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>2</v>
       </c>
@@ -3716,7 +3849,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>2</v>
       </c>
@@ -3757,7 +3890,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -3795,7 +3928,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -3833,7 +3966,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -3868,7 +4001,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>2</v>
       </c>
@@ -3900,7 +4033,7 @@
         <v>3.6296296296296298</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -3932,7 +4065,7 @@
         <v>3.1111111111111112</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -3964,7 +4097,7 @@
         <v>2.9629629629629624</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -3996,7 +4129,7 @@
         <v>2.4444444444444446</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>2</v>
       </c>
@@ -4028,7 +4161,7 @@
         <v>1.7037037037037035</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -4066,7 +4199,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -4104,7 +4237,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -4142,7 +4275,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -4180,7 +4313,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>2</v>
       </c>
@@ -4215,7 +4348,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -4250,7 +4383,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>2</v>
       </c>
@@ -4291,7 +4424,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>2</v>
       </c>
@@ -4329,7 +4462,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>2</v>
       </c>
@@ -4367,7 +4500,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -4408,7 +4541,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -4449,7 +4582,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -4487,7 +4620,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -4525,7 +4658,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>2</v>
       </c>
@@ -4563,7 +4696,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -4599,7 +4732,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>2</v>
       </c>
@@ -4635,7 +4768,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>2</v>
       </c>
@@ -4671,7 +4804,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>2</v>
       </c>
@@ -4706,7 +4839,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>2</v>
       </c>
@@ -4738,7 +4871,7 @@
         <v>3.1111111111111112</v>
       </c>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>2</v>
       </c>
@@ -4770,7 +4903,7 @@
         <v>2.9629629629629624</v>
       </c>
     </row>
-    <row r="57" spans="1:13">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>2</v>
       </c>
@@ -4802,7 +4935,7 @@
         <v>2.4444444444444446</v>
       </c>
     </row>
-    <row r="58" spans="1:13">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>2</v>
       </c>
@@ -4834,7 +4967,7 @@
         <v>1.7037037037037035</v>
       </c>
     </row>
-    <row r="59" spans="1:13">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>2</v>
       </c>
@@ -4871,7 +5004,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="60" spans="1:13">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>2</v>
       </c>
@@ -4903,7 +5036,7 @@
         <v>0.96573208722741399</v>
       </c>
     </row>
-    <row r="61" spans="1:13">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>2</v>
       </c>
@@ -4935,7 +5068,7 @@
         <v>0.9785932721712538</v>
       </c>
     </row>
-    <row r="62" spans="1:13">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>2</v>
       </c>
@@ -4967,7 +5100,7 @@
         <v>0.98084677419354838</v>
       </c>
     </row>
-    <row r="63" spans="1:13">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>2</v>
       </c>
@@ -4999,7 +5132,7 @@
         <v>0.98884381338742389</v>
       </c>
     </row>
-    <row r="64" spans="1:13">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>2</v>
       </c>
@@ -5031,7 +5164,7 @@
         <v>0.98377281947261663</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="57.75">
+    <row r="65" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>3</v>
       </c>
@@ -5066,7 +5199,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="15">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -5098,7 +5231,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="43.5">
+    <row r="67" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>2</v>
       </c>
@@ -5134,7 +5267,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="43.5">
+    <row r="68" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>2</v>
       </c>
@@ -5170,7 +5303,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="43.5">
+    <row r="69" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -5206,7 +5339,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="43.5">
+    <row r="70" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>2</v>
       </c>
@@ -5242,7 +5375,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="43.5">
+    <row r="71" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>2</v>
       </c>
@@ -5278,7 +5411,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="43.5">
+    <row r="72" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>2</v>
       </c>
@@ -5314,7 +5447,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="29.25">
+    <row r="73" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>2</v>
       </c>
@@ -5346,7 +5479,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="74" spans="1:13">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>2</v>
       </c>
@@ -5375,7 +5508,7 @@
         <v>0.33600000000000002</v>
       </c>
     </row>
-    <row r="75" spans="1:13">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>2</v>
       </c>
@@ -5404,7 +5537,7 @@
         <v>0.44800000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:13">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>2</v>
       </c>
@@ -5433,7 +5566,7 @@
         <v>0.54600000000000004</v>
       </c>
     </row>
-    <row r="77" spans="1:13">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>2</v>
       </c>
@@ -5462,7 +5595,7 @@
         <v>0.63300000000000001</v>
       </c>
     </row>
-    <row r="78" spans="1:13">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -5491,7 +5624,7 @@
         <v>0.67600000000000005</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="29.25">
+    <row r="79" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>2</v>
       </c>
@@ -5527,7 +5660,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="80" spans="1:13">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>2</v>
       </c>
@@ -5560,7 +5693,7 @@
         <v>24.814814814814813</v>
       </c>
     </row>
-    <row r="81" spans="1:13">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>2</v>
       </c>
@@ -5593,7 +5726,7 @@
         <v>33.333333333333336</v>
       </c>
     </row>
-    <row r="82" spans="1:13">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>2</v>
       </c>
@@ -5626,7 +5759,7 @@
         <v>35.037037037037031</v>
       </c>
     </row>
-    <row r="83" spans="1:13">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>2</v>
       </c>
@@ -5659,7 +5792,7 @@
         <v>37.777777777777779</v>
       </c>
     </row>
-    <row r="84" spans="1:13">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>2</v>
       </c>
@@ -5692,7 +5825,7 @@
         <v>39.037037037037031</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="43.5">
+    <row r="85" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>2</v>
       </c>
@@ -5728,7 +5861,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="86" spans="1:13" ht="43.5">
+    <row r="86" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>2</v>
       </c>
@@ -5764,7 +5897,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="43.5">
+    <row r="87" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>2</v>
       </c>
@@ -5800,7 +5933,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="88" spans="1:13">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>2</v>
       </c>
@@ -5835,7 +5968,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="89" spans="1:13">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>2</v>
       </c>
@@ -5867,7 +6000,7 @@
         <v>23.475200000000001</v>
       </c>
     </row>
-    <row r="90" spans="1:13">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>2</v>
       </c>
@@ -5899,7 +6032,7 @@
         <v>33.142200000000003</v>
       </c>
     </row>
-    <row r="91" spans="1:13">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>2</v>
       </c>
@@ -5931,7 +6064,7 @@
         <v>46.652100000000004</v>
       </c>
     </row>
-    <row r="92" spans="1:13">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>2</v>
       </c>
@@ -5963,7 +6096,7 @@
         <v>53.742000000000004</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="29.25">
+    <row r="93" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>2</v>
       </c>
@@ -5999,7 +6132,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="94" spans="1:13" ht="29.25">
+    <row r="94" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>2</v>
       </c>
@@ -6035,7 +6168,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="95" spans="1:13" ht="29.25">
+    <row r="95" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>2</v>
       </c>
@@ -6071,7 +6204,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="96" spans="1:13">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>2</v>
       </c>
@@ -6107,7 +6240,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="97" spans="1:13">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>2</v>
       </c>
@@ -6140,7 +6273,7 @@
         <v>33.333333333333336</v>
       </c>
     </row>
-    <row r="98" spans="1:13">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>2</v>
       </c>
@@ -6173,7 +6306,7 @@
         <v>35.037037037037031</v>
       </c>
     </row>
-    <row r="99" spans="1:13">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>2</v>
       </c>
@@ -6206,7 +6339,7 @@
         <v>37.777777777777779</v>
       </c>
     </row>
-    <row r="100" spans="1:13">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>2</v>
       </c>
@@ -6239,7 +6372,7 @@
         <v>39.037037037037031</v>
       </c>
     </row>
-    <row r="101" spans="1:13" ht="29.25">
+    <row r="101" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>2</v>
       </c>
@@ -6271,7 +6404,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="102" spans="1:13">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>2</v>
       </c>
@@ -6300,7 +6433,7 @@
         <v>0.33600000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:13">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>2</v>
       </c>
@@ -6329,7 +6462,7 @@
         <v>0.44800000000000001</v>
       </c>
     </row>
-    <row r="104" spans="1:13">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>2</v>
       </c>
@@ -6358,7 +6491,7 @@
         <v>0.54600000000000004</v>
       </c>
     </row>
-    <row r="105" spans="1:13">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>2</v>
       </c>
@@ -6387,7 +6520,7 @@
         <v>0.63300000000000001</v>
       </c>
     </row>
-    <row r="106" spans="1:13">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>2</v>
       </c>
@@ -6456,17 +6589,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC50408-61D8-4A10-93E8-9867356C2F54}">
   <dimension ref="A1:Q8"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="17" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.54296875" customWidth="1"/>
+    <col min="6" max="6" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="17" width="15.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -6493,7 +6626,7 @@
       <c r="P1" s="34"/>
       <c r="Q1" s="34"/>
     </row>
-    <row r="2" spans="1:17" ht="15">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -6522,7 +6655,7 @@
       <c r="P2" s="33"/>
       <c r="Q2" s="33"/>
     </row>
-    <row r="3" spans="1:17" ht="15">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>89</v>
       </c>
@@ -6559,7 +6692,7 @@
       </c>
       <c r="Q3" s="33"/>
     </row>
-    <row r="4" spans="1:17" ht="15">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -6612,7 +6745,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -6623,7 +6756,7 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:17" ht="15">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>92</v>
       </c>
@@ -6678,7 +6811,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>95</v>
       </c>
@@ -6735,7 +6868,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -6827,18 +6960,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC26D125-533B-4E2C-8B10-83B96EF6CBCB}">
   <dimension ref="A1:L25"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="50.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="50.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6876,7 +7009,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -6905,7 +7038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -6934,7 +7067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -6966,7 +7099,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -6998,7 +7131,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -7030,7 +7163,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -7062,7 +7195,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -7094,7 +7227,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -7124,7 +7257,7 @@
       </c>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -7154,7 +7287,7 @@
       </c>
       <c r="L10" s="9"/>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -7184,7 +7317,7 @@
       </c>
       <c r="L11" s="9"/>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -7214,7 +7347,7 @@
       </c>
       <c r="L12" s="9"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -7244,7 +7377,7 @@
       </c>
       <c r="L13" s="9"/>
     </row>
-    <row r="14" spans="1:12" ht="101.45">
+    <row r="14" spans="1:12" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -7276,7 +7409,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -7308,7 +7441,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -7338,7 +7471,7 @@
       </c>
       <c r="L16" s="9"/>
     </row>
-    <row r="17" spans="1:12" ht="43.5">
+    <row r="17" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -7370,7 +7503,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="43.5">
+    <row r="18" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -7402,7 +7535,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -7434,7 +7567,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -7466,7 +7599,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -7495,7 +7628,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -7524,7 +7657,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>1</v>
       </c>
@@ -7553,7 +7686,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -7582,7 +7715,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -7646,16 +7779,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B8AA13D-2CC0-4240-A9BF-02BB80A27D5D}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.26953125" customWidth="1"/>
+    <col min="4" max="4" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -7675,7 +7808,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -7698,7 +7831,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -7706,7 +7839,7 @@
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>110</v>
       </c>
@@ -7729,7 +7862,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>114</v>
       </c>
@@ -7758,7 +7891,7 @@
         <v>Missing</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>115</v>
       </c>
@@ -7787,7 +7920,7 @@
         <v>Missing</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>116</v>
       </c>
@@ -7810,7 +7943,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>117</v>
       </c>
@@ -7833,7 +7966,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>118</v>
       </c>
@@ -7859,7 +7992,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>120</v>
       </c>
@@ -7887,7 +8020,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>122</v>
       </c>
@@ -7914,7 +8047,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -7937,7 +8070,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -7963,7 +8096,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>127</v>
       </c>
@@ -7989,7 +8122,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>129</v>
       </c>
@@ -8033,16 +8166,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F427D668-6E74-4989-9A76-CA42E7F92A98}">
   <dimension ref="A1:J76"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.42578125" customWidth="1"/>
+    <col min="3" max="3" width="40.453125" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="7" max="7" width="34.140625" customWidth="1"/>
-    <col min="10" max="10" width="50.42578125" customWidth="1"/>
+    <col min="7" max="7" width="34.1796875" customWidth="1"/>
+    <col min="10" max="10" width="50.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8074,7 +8207,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.95">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -8094,7 +8227,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="32.25" customHeight="1">
+    <row r="3" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -8114,7 +8247,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -8131,7 +8264,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -8148,7 +8281,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -8165,7 +8298,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -8182,7 +8315,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>135</v>
       </c>
@@ -8199,7 +8332,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>135</v>
       </c>
@@ -8216,7 +8349,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>135</v>
       </c>
@@ -8233,7 +8366,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -8250,7 +8383,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>135</v>
       </c>
@@ -8267,7 +8400,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>135</v>
       </c>
@@ -8284,7 +8417,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -8301,7 +8434,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>3</v>
       </c>
@@ -8318,7 +8451,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>3</v>
       </c>
@@ -8335,7 +8468,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -8352,7 +8485,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -8369,7 +8502,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -8386,7 +8519,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15.95">
+    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -8406,7 +8539,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>1</v>
       </c>
@@ -8426,7 +8559,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -8443,7 +8576,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>1</v>
       </c>
@@ -8460,7 +8593,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>1</v>
       </c>
@@ -8477,7 +8610,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -8494,7 +8627,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>135</v>
       </c>
@@ -8511,7 +8644,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>135</v>
       </c>
@@ -8528,7 +8661,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>135</v>
       </c>
@@ -8545,7 +8678,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>135</v>
       </c>
@@ -8562,7 +8695,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>135</v>
       </c>
@@ -8579,7 +8712,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>135</v>
       </c>
@@ -8596,7 +8729,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -8613,7 +8746,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>3</v>
       </c>
@@ -8630,7 +8763,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>3</v>
       </c>
@@ -8647,7 +8780,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -8664,7 +8797,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -8681,7 +8814,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>3</v>
       </c>
@@ -8698,7 +8831,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>1</v>
       </c>
@@ -8712,7 +8845,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -8726,7 +8859,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -8740,7 +8873,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>1</v>
       </c>
@@ -8754,7 +8887,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>1</v>
       </c>
@@ -8768,7 +8901,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>1</v>
       </c>
@@ -8782,7 +8915,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>135</v>
       </c>
@@ -8796,7 +8929,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>135</v>
       </c>
@@ -8810,7 +8943,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>135</v>
       </c>
@@ -8824,7 +8957,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>135</v>
       </c>
@@ -8838,7 +8971,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>135</v>
       </c>
@@ -8852,7 +8985,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>135</v>
       </c>
@@ -8866,7 +8999,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -8880,7 +9013,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -8894,7 +9027,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -8908,7 +9041,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -8922,7 +9055,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -8936,7 +9069,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -8950,7 +9083,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -8964,7 +9097,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="43.5">
+    <row r="57" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>1</v>
       </c>
@@ -8978,7 +9111,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15.95">
+    <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -8992,7 +9125,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15.95">
+    <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>1</v>
       </c>
@@ -9004,7 +9137,7 @@
       </c>
       <c r="J59" s="12"/>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>1</v>
       </c>
@@ -9015,7 +9148,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>1</v>
       </c>
@@ -9026,7 +9159,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>135</v>
       </c>
@@ -9040,7 +9173,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>135</v>
       </c>
@@ -9051,7 +9184,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>135</v>
       </c>
@@ -9062,7 +9195,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>135</v>
       </c>
@@ -9073,7 +9206,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>135</v>
       </c>
@@ -9084,7 +9217,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>135</v>
       </c>
@@ -9095,7 +9228,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>3</v>
       </c>
@@ -9109,7 +9242,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>3</v>
       </c>
@@ -9120,7 +9253,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>3</v>
       </c>
@@ -9131,7 +9264,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>3</v>
       </c>
@@ -9142,7 +9275,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>3</v>
       </c>
@@ -9153,7 +9286,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>3</v>
       </c>
@@ -9164,7 +9297,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="29.45">
+    <row r="74" spans="1:10" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>1</v>
       </c>
@@ -9184,7 +9317,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>135</v>
       </c>
@@ -9201,7 +9334,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>3</v>
       </c>
@@ -9254,15 +9387,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E519DD-7070-48BB-9F21-242D1E473943}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -9279,14 +9412,14 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>154</v>
       </c>
@@ -9302,7 +9435,7 @@
         <v>Complete</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
         <v>155</v>
       </c>
@@ -9331,18 +9464,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BE8E890-3EB7-493D-B8C3-05E861B2DBA4}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="6" max="6" width="34.140625" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="50.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.26953125" customWidth="1"/>
+    <col min="6" max="6" width="34.1796875" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="50.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -9371,7 +9504,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="101.45">
+    <row r="2" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -9400,7 +9533,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -9429,7 +9562,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -9458,7 +9591,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -9487,7 +9620,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -9548,15 +9681,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{259F6A5D-CF80-41BD-979A-295E7564EADB}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="56.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="150" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -9583,7 +9716,7 @@
       </c>
       <c r="I1" s="23"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
         <v>172</v>
       </c>
@@ -9596,7 +9729,7 @@
       <c r="H2" s="23"/>
       <c r="I2" s="23"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>173</v>
       </c>
@@ -9623,7 +9756,7 @@
       </c>
       <c r="I3" s="23"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
         <v>179</v>
       </c>
@@ -9648,7 +9781,7 @@
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
         <v>184</v>
       </c>
@@ -9661,7 +9794,7 @@
       <c r="H5" s="23"/>
       <c r="I5" s="23"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="26" t="s">
         <v>185</v>
       </c>
@@ -9680,7 +9813,7 @@
       <c r="H6" s="23"/>
       <c r="I6" s="23"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
         <v>185</v>
       </c>
@@ -9699,7 +9832,7 @@
       <c r="H7" s="23"/>
       <c r="I7" s="23"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="26" t="s">
         <v>191</v>
       </c>
@@ -9720,7 +9853,7 @@
       </c>
       <c r="I8" s="23"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
@@ -9731,7 +9864,7 @@
       <c r="H9" s="23"/>
       <c r="I9" s="23"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
@@ -9742,7 +9875,7 @@
       <c r="H10" s="23"/>
       <c r="I10" s="23"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="23"/>
@@ -9753,7 +9886,7 @@
       <c r="H11" s="23"/>
       <c r="I11" s="23"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="23"/>
@@ -9764,7 +9897,7 @@
       <c r="H12" s="23"/>
       <c r="I12" s="23"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="23"/>
@@ -9775,7 +9908,7 @@
       <c r="H13" s="23"/>
       <c r="I13" s="23"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="23"/>
@@ -9795,14 +9928,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10060,22 +10191,51 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="19a3940c-c740-4699-845a-46837f99845a"/>
+    <ds:schemaRef ds:uri="539a68f6-d0ac-4a73-9041-e1fa437c4cee"/>
+    <ds:schemaRef ds:uri="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a"/>
+    <ds:schemaRef ds:uri="19a3940c-c740-4699-845a-46837f99845a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changes for Nigeria Scenarios
Bouillon required no changes
Rice has an increase in Vehicle "fortifiability" based on a calculation from BCG.
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\projects\2026\vivarium_gates_lsff_2026\0100_data_prep\extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39FB672-C793-48C2-A2AD-70ED8B1DFACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDD5D43-72C8-4624-AEAC-2BD6AB93517F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Country-Vehicle Progress" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,10 @@
     <sheet name="Scenario Definition Extraction" sheetId="15" r:id="rId11"/>
     <sheet name="Data Sources" sheetId="8" r:id="rId12"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Country-Vehicle Extraction'!$A$1:$M$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Scenario Definition Extraction'!$A$1:$J$28</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -47,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="238">
   <si>
     <t>Country</t>
   </si>
@@ -457,7 +461,7 @@
       <rPr>
         <sz val="12"/>
         <rFont val="Aptos"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t>  </t>
     </r>
@@ -482,7 +486,7 @@
       <rPr>
         <sz val="12"/>
         <rFont val="Aptos"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t> </t>
     </r>
@@ -780,6 +784,12 @@
   </si>
   <si>
     <t>Kept consistent with the existing NRV scenarios so the three arms differ only in concentration. GF Apr-2026 workbook implies 2030 compliance = 80% (effectiveness 1.0 at 0.8 reach); to be adopted for all Ethiopia scenarios together in the parameter-update batch.</t>
+  </si>
+  <si>
+    <t>"Updated for Portfolio Review - 3.92 / 5.23 MT" and is attributed to Laura Key (Boston Consulting Group), from "20260416_Input data to IHME models.xlsx" and on both the "Vehicles - WRA" and "Vehicles - Preschool" sheets, cell Q10</t>
+  </si>
+  <si>
+    <t>BCG-measured tonnage</t>
   </si>
 </sst>
 </file>
@@ -811,6 +821,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -840,40 +851,41 @@
       <sz val="11"/>
       <color rgb="FF444444"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Aptos"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Aptos"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -881,12 +893,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -894,6 +908,7 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -901,6 +916,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1928,7 +1944,7 @@
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:J8 B6:C8">
+  <conditionalFormatting sqref="B6:C8 E6:J8">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Missing"</formula>
     </cfRule>
@@ -2812,6 +2828,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J28" xr:uid="{797B3B46-8F2E-4C67-A115-D7583B1B84DB}"/>
   <dataValidations count="4">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:B1" xr:uid="{998163E2-1EA2-4797-843A-F967F70AD818}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1048576" xr:uid="{FB33DD5A-6B57-46A5-BB2A-AA6288CEC89B}">
@@ -2831,6 +2848,7 @@
     <hyperlink ref="J23" r:id="rId4" xr:uid="{E1E2866D-3A5C-4D33-8B50-C6AA8A296518}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -5222,13 +5240,13 @@
         <v>30</v>
       </c>
       <c r="I66" t="s">
-        <v>47</v>
+        <v>237</v>
       </c>
       <c r="J66" s="7">
-        <v>0.3</v>
-      </c>
-      <c r="M66" s="5" t="s">
-        <v>82</v>
+        <v>0.74</v>
+      </c>
+      <c r="M66" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -6550,6 +6568,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M106" xr:uid="{4F7501F0-08E1-4A63-A382-F6741C91E79A}"/>
   <dataValidations count="5">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:B1" xr:uid="{E441A666-11EF-40F7-A6AA-2528D8D84D13}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{01C8494E-7753-4018-8855-0065C3105F7C}">
@@ -9928,15 +9947,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -10190,6 +10200,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -10202,14 +10221,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10229,6 +10240,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44149C33-81B0-4C8D-A8B9-4C0F99EB683B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Changes for India scenarios
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\projects\2026\vivarium_gates_lsff_2026\0100_data_prep\extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDD5D43-72C8-4624-AEAC-2BD6AB93517F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08002D3-F155-4A73-93BA-5F78F877EE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Country-Vehicle Progress" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="240">
   <si>
     <t>Country</t>
   </si>
@@ -294,9 +294,6 @@
   </si>
   <si>
     <t>Table 169, page 220 'Percentage of Non-Pregnant Women Whose Households Consumed Bouillon (purchased, branded, and labelled as fortified) by Residence, Zone, and Wealth Quintile', using 'branded' as a proxy for fortifiable and % of households as a proxy for % of product. Values obtained by dividing percent consuming branded food by percent consuming food, which is why we don't have uncertainty. A similar thing is reported in Annex 43, page 549; 'How household obtained bouillon the last time it was obtained': 'purchased', and not by wealth quintile</t>
-  </si>
-  <si>
-    <t>51.3% "Industry consolidation" sent by Jonathan Gorstein in a spreadsheet on 7/19 according to M4N Database, but on 8/15 we agreed to consider all open-market rice unfortifiable</t>
   </si>
   <si>
     <t>Jonathan Gorstein email 8/30</t>
@@ -790,6 +787,15 @@
   </si>
   <si>
     <t>BCG-measured tonnage</t>
+  </si>
+  <si>
+    <t>51.3% "Industry consolidation" sent by Jonathan Gorstein in a spreadsheet on 7/19/2024 according to M4N Database, but on 8/15/2024 we agreed to consider all open-market rice unfortifiable; in 2025 or 26 Laura Key (Boston Consulting Group) put 45% in the "Vehicles - preschool" sheet entry for India Rice Industry consolidation</t>
+  </si>
+  <si>
+    <t>"20260416_Input data to IHME models.xlsx" Compliance projection for 2030</t>
+  </si>
+  <si>
+    <t>Laura Key (BCG), "India_Bangladesh_data" (note in "Vehicles - preschool!Q48" of "20260416_Input data to IHME models.xlsx"</t>
   </si>
 </sst>
 </file>
@@ -947,7 +953,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1007,6 +1013,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1746,62 +1753,62 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>89</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>90</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
       <c r="E3" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="F3" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="F3" s="28" t="s">
-        <v>91</v>
-      </c>
       <c r="G3" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="H3" s="28" t="s">
-        <v>91</v>
-      </c>
       <c r="I3" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="J3" s="28" t="s">
         <v>90</v>
-      </c>
-      <c r="J3" s="28" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="31" t="s">
         <v>195</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="C4" s="31" t="s">
         <v>196</v>
       </c>
-      <c r="C4" s="31" t="s">
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E4" s="31" t="s">
         <v>197</v>
       </c>
-      <c r="D4" t="s">
-        <v>229</v>
-      </c>
-      <c r="E4" s="31" t="s">
-        <v>198</v>
-      </c>
       <c r="F4" s="31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I4" s="31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J4" s="31" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -1815,7 +1822,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B6" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
@@ -1826,7 +1833,7 @@
         <v>Complete</v>
       </c>
       <c r="D6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E6" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A6) = 0, "Missing", "Complete")</f>
@@ -1855,7 +1862,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B7" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
@@ -1866,7 +1873,7 @@
         <v>Complete</v>
       </c>
       <c r="D7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E7" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A7) = 0, "Missing", "Complete")</f>
@@ -1895,7 +1902,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B8" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, B$1,  'Scenario Definition Extraction'!$B$2:$B$1000, B$2,  'Scenario Definition Extraction'!$C$2:$C$1000, B$3, 'Scenario Definition Extraction'!$D$2:$D$1000, B$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
@@ -1906,7 +1913,7 @@
         <v>Complete</v>
       </c>
       <c r="D8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E8" t="str">
         <f>IF(COUNTIFS('Scenario Definition Extraction'!$A$2:$A$1000, E$1,  'Scenario Definition Extraction'!$B$2:$B$1000, E$2,  'Scenario Definition Extraction'!$C$2:$C$1000, E$3, 'Scenario Definition Extraction'!$D$2:$D$1000, E$4, 'Scenario Definition Extraction'!$E$2:$E$1000, $A8) = 0, "Missing", "Complete")</f>
@@ -1975,10 +1982,10 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>11</v>
@@ -2007,13 +2014,13 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
@@ -2022,7 +2029,7 @@
         <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I2" s="7">
         <v>0.9</v>
@@ -2036,13 +2043,13 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -2051,7 +2058,7 @@
         <v>30</v>
       </c>
       <c r="H3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I3" s="7">
         <v>0.9</v>
@@ -2065,13 +2072,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
@@ -2080,7 +2087,7 @@
         <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I4" s="7">
         <v>0.9</v>
@@ -2094,13 +2101,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F5" t="s">
         <v>29</v>
@@ -2109,7 +2116,7 @@
         <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I5" s="7">
         <v>0.9</v>
@@ -2123,13 +2130,13 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F6" t="s">
         <v>29</v>
@@ -2138,13 +2145,13 @@
         <v>30</v>
       </c>
       <c r="H6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I6" s="7">
         <v>0.8</v>
       </c>
       <c r="J6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -2155,13 +2162,13 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F7" t="s">
         <v>29</v>
@@ -2170,13 +2177,13 @@
         <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I7" s="7">
         <v>0.8</v>
       </c>
       <c r="J7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -2187,13 +2194,13 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
@@ -2202,13 +2209,13 @@
         <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I8" s="7">
         <v>0.8</v>
       </c>
       <c r="J8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -2219,13 +2226,13 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -2234,13 +2241,13 @@
         <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I9" s="7">
         <v>0.8</v>
       </c>
       <c r="J9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -2251,13 +2258,13 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -2266,13 +2273,13 @@
         <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I10" s="7">
         <v>0.8</v>
       </c>
       <c r="J10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -2283,13 +2290,13 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -2298,7 +2305,7 @@
         <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I11" s="7">
         <v>0.9</v>
@@ -2312,13 +2319,13 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E12" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
@@ -2327,7 +2334,7 @@
         <v>30</v>
       </c>
       <c r="H12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I12" s="7">
         <v>0.9</v>
@@ -2341,13 +2348,13 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -2356,7 +2363,7 @@
         <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I13" s="7">
         <v>0.9</v>
@@ -2370,13 +2377,13 @@
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F14" t="s">
         <v>29</v>
@@ -2385,7 +2392,7 @@
         <v>30</v>
       </c>
       <c r="H14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I14" s="7">
         <v>0.9</v>
@@ -2399,13 +2406,13 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
@@ -2414,7 +2421,7 @@
         <v>30</v>
       </c>
       <c r="H15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I15" s="7">
         <v>0.9</v>
@@ -2428,13 +2435,13 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D16" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F16" t="s">
         <v>29</v>
@@ -2443,7 +2450,7 @@
         <v>30</v>
       </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I16" s="7">
         <v>0.9</v>
@@ -2457,13 +2464,13 @@
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
@@ -2472,13 +2479,13 @@
         <v>30</v>
       </c>
       <c r="H17" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I17" s="7">
         <v>0.9</v>
       </c>
       <c r="J17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -2489,13 +2496,13 @@
         <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E18" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
@@ -2504,10 +2511,10 @@
         <v>30</v>
       </c>
       <c r="H18" t="s">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="I18" s="7">
-        <v>0.8</v>
+        <v>0.9375</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -2518,13 +2525,13 @@
         <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E19" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -2533,10 +2540,10 @@
         <v>30</v>
       </c>
       <c r="H19" t="s">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="I19" s="7">
-        <v>0.8</v>
+        <v>0.9375</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2547,28 +2554,28 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D20" t="s">
+        <v>197</v>
+      </c>
+      <c r="E20" t="s">
         <v>198</v>
       </c>
-      <c r="E20" t="s">
-        <v>199</v>
-      </c>
       <c r="F20" t="s">
+        <v>97</v>
+      </c>
+      <c r="G20" t="s">
         <v>98</v>
       </c>
-      <c r="G20" t="s">
-        <v>99</v>
-      </c>
       <c r="H20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I20">
         <v>1320</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2579,28 +2586,28 @@
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D21" t="s">
+        <v>197</v>
+      </c>
+      <c r="E21" t="s">
         <v>198</v>
       </c>
-      <c r="E21" t="s">
-        <v>199</v>
-      </c>
       <c r="F21" t="s">
+        <v>97</v>
+      </c>
+      <c r="G21" t="s">
         <v>98</v>
       </c>
-      <c r="G21" t="s">
-        <v>99</v>
-      </c>
       <c r="H21" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I21">
         <v>24</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -2611,28 +2618,28 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D22" t="s">
+        <v>197</v>
+      </c>
+      <c r="E22" t="s">
         <v>198</v>
       </c>
-      <c r="E22" t="s">
-        <v>199</v>
-      </c>
       <c r="F22" t="s">
+        <v>97</v>
+      </c>
+      <c r="G22" t="s">
         <v>98</v>
       </c>
-      <c r="G22" t="s">
-        <v>99</v>
-      </c>
       <c r="H22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I22">
         <v>40</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -2643,28 +2650,28 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E23" t="s">
         <v>198</v>
       </c>
-      <c r="E23" t="s">
-        <v>199</v>
-      </c>
       <c r="F23" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" t="s">
         <v>98</v>
       </c>
-      <c r="G23" t="s">
-        <v>99</v>
-      </c>
       <c r="H23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I23">
         <v>1.69</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -2675,28 +2682,28 @@
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D24" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E24" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F24" t="s">
+        <v>97</v>
+      </c>
+      <c r="G24" t="s">
         <v>98</v>
       </c>
-      <c r="G24" t="s">
-        <v>99</v>
-      </c>
       <c r="H24" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I24">
         <v>14.084507042253522</v>
       </c>
       <c r="J24" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -2707,28 +2714,28 @@
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D25" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F25" t="s">
+        <v>97</v>
+      </c>
+      <c r="G25" t="s">
         <v>98</v>
       </c>
-      <c r="G25" t="s">
-        <v>99</v>
-      </c>
       <c r="H25" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I25">
         <v>56.338028169014088</v>
       </c>
       <c r="J25" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -2739,28 +2746,28 @@
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D26" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E26" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F26" t="s">
+        <v>97</v>
+      </c>
+      <c r="G26" t="s">
         <v>98</v>
       </c>
-      <c r="G26" t="s">
-        <v>99</v>
-      </c>
       <c r="H26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I26">
         <v>45</v>
       </c>
       <c r="J26" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -2771,28 +2778,28 @@
         <v>7</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
+        <v>197</v>
+      </c>
+      <c r="E27" t="s">
         <v>198</v>
       </c>
-      <c r="E27" t="s">
-        <v>199</v>
-      </c>
       <c r="F27" t="s">
+        <v>97</v>
+      </c>
+      <c r="G27" t="s">
         <v>98</v>
       </c>
-      <c r="G27" t="s">
-        <v>99</v>
-      </c>
       <c r="H27" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I27">
         <v>42.5</v>
       </c>
       <c r="J27" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
@@ -2803,28 +2810,28 @@
         <v>7</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D28" t="s">
+        <v>197</v>
+      </c>
+      <c r="E28" t="s">
         <v>198</v>
       </c>
-      <c r="E28" t="s">
-        <v>199</v>
-      </c>
       <c r="F28" t="s">
+        <v>97</v>
+      </c>
+      <c r="G28" t="s">
         <v>98</v>
       </c>
-      <c r="G28" t="s">
-        <v>99</v>
-      </c>
       <c r="H28" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="I28">
         <v>1.3</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2882,22 +2889,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
@@ -2905,13 +2912,13 @@
         <v>49</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E2">
         <v>2021</v>
@@ -2919,30 +2926,30 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B3" t="s">
         <v>221</v>
-      </c>
-      <c r="B3" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B4" t="s">
         <v>223</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" t="s">
         <v>225</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" t="s">
         <v>227</v>
-      </c>
-      <c r="F4" t="s">
-        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -5182,7 +5189,7 @@
         <v>0.98377281947261663</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" ht="87" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>3</v>
       </c>
@@ -5207,14 +5214,14 @@
       <c r="H65">
         <v>2024</v>
       </c>
-      <c r="I65" t="s">
-        <v>47</v>
+      <c r="I65" s="35" t="s">
+        <v>239</v>
       </c>
       <c r="J65" s="21">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="M65" s="5" t="s">
-        <v>81</v>
+        <v>237</v>
       </c>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.35">
@@ -5240,13 +5247,13 @@
         <v>30</v>
       </c>
       <c r="I66" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J66" s="7">
         <v>0.74</v>
       </c>
       <c r="M66" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5282,7 +5289,7 @@
         <v>32.803200000000004</v>
       </c>
       <c r="M67" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5318,7 +5325,7 @@
         <v>11.491200000000001</v>
       </c>
       <c r="M68" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5354,7 +5361,7 @@
         <v>23.475200000000001</v>
       </c>
       <c r="M69" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5390,7 +5397,7 @@
         <v>33.142200000000003</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5426,7 +5433,7 @@
         <v>46.652100000000004</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5462,7 +5469,7 @@
         <v>53.742000000000004</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="29" x14ac:dyDescent="0.35">
@@ -5488,13 +5495,13 @@
         <v>30</v>
       </c>
       <c r="I73" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J73" s="21">
         <v>0.53600000000000003</v>
       </c>
       <c r="M73" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.35">
@@ -5520,7 +5527,7 @@
         <v>30</v>
       </c>
       <c r="I74" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J74" s="21">
         <v>0.33600000000000002</v>
@@ -5549,7 +5556,7 @@
         <v>30</v>
       </c>
       <c r="I75" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J75" s="21">
         <v>0.44800000000000001</v>
@@ -5578,7 +5585,7 @@
         <v>30</v>
       </c>
       <c r="I76" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J76" s="21">
         <v>0.54600000000000004</v>
@@ -5607,7 +5614,7 @@
         <v>30</v>
       </c>
       <c r="I77" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J77" s="21">
         <v>0.63300000000000001</v>
@@ -5636,7 +5643,7 @@
         <v>30</v>
       </c>
       <c r="I78" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J78" s="21">
         <v>0.67600000000000005</v>
@@ -5675,7 +5682,7 @@
         <v>40.074074074074069</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.35">
@@ -5876,7 +5883,7 @@
         <v>20.5288</v>
       </c>
       <c r="M85" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5912,7 +5919,7 @@
         <v>19.028000000000002</v>
       </c>
       <c r="M86" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="87" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
@@ -5948,7 +5955,7 @@
         <v>21.976000000000003</v>
       </c>
       <c r="M87" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.35">
@@ -6147,7 +6154,7 @@
         <v>25.62962962962963</v>
       </c>
       <c r="M93" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="94" spans="1:13" ht="29" x14ac:dyDescent="0.35">
@@ -6183,7 +6190,7 @@
         <v>23.999999999999996</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="95" spans="1:13" ht="29" x14ac:dyDescent="0.35">
@@ -6219,7 +6226,7 @@
         <v>27.333333333333336</v>
       </c>
       <c r="M95" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.35">
@@ -6413,13 +6420,13 @@
         <v>30</v>
       </c>
       <c r="I101" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J101" s="21">
         <v>0.53600000000000003</v>
       </c>
       <c r="M101" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.35">
@@ -6445,7 +6452,7 @@
         <v>30</v>
       </c>
       <c r="I102" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J102" s="21">
         <v>0.33600000000000002</v>
@@ -6474,7 +6481,7 @@
         <v>30</v>
       </c>
       <c r="I103" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J103" s="21">
         <v>0.44800000000000001</v>
@@ -6503,7 +6510,7 @@
         <v>30</v>
       </c>
       <c r="I104" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J104" s="21">
         <v>0.54600000000000004</v>
@@ -6532,7 +6539,7 @@
         <v>30</v>
       </c>
       <c r="I105" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J105" s="21">
         <v>0.63300000000000001</v>
@@ -6561,7 +6568,7 @@
         <v>30</v>
       </c>
       <c r="I106" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J106" s="21">
         <v>0.67600000000000005</v>
@@ -6590,6 +6597,7 @@
     <hyperlink ref="M17" r:id="rId3" xr:uid="{1650080F-1085-40E4-8BD5-886F921DD675}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
@@ -6676,38 +6684,38 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>89</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>90</v>
       </c>
       <c r="C3" s="33"/>
       <c r="D3" s="33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E3" s="33"/>
       <c r="F3" s="33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G3" s="33"/>
       <c r="H3" s="33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I3" s="33"/>
       <c r="J3" s="33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K3" s="33"/>
       <c r="L3" s="33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M3" s="33"/>
       <c r="N3" s="33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O3" s="33"/>
       <c r="P3" s="33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q3" s="33"/>
     </row>
@@ -6777,25 +6785,25 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" t="s">
         <v>92</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" t="s">
         <v>93</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>93</v>
       </c>
-      <c r="D6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E6" t="s">
-        <v>94</v>
-      </c>
       <c r="F6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H6" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A6, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -6806,16 +6814,16 @@
         <v>Complete</v>
       </c>
       <c r="J6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N6" t="s">
         <v>13</v>
@@ -6832,25 +6840,25 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" t="s">
         <v>93</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>93</v>
       </c>
-      <c r="D7" t="s">
-        <v>94</v>
-      </c>
-      <c r="E7" t="s">
-        <v>94</v>
-      </c>
       <c r="F7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -6861,53 +6869,53 @@
         <v>Missing</v>
       </c>
       <c r="J7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, N$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="O7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P7" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, P$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A7, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="Q7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" t="s">
         <v>93</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>93</v>
       </c>
-      <c r="D8" t="s">
-        <v>94</v>
-      </c>
-      <c r="E8" t="s">
-        <v>94</v>
-      </c>
       <c r="F8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, F$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, F$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, H$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "Total",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
@@ -6918,30 +6926,30 @@
         <v>Missing</v>
       </c>
       <c r="J8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, N$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="O8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P8" t="str">
         <f>IF(COUNTIFS('Country-Vehicle-Fort Extraction'!$A$2:$A$944, N$1,  'Country-Vehicle-Fort Extraction'!$B$2:$B$944, N$2,  'Country-Vehicle-Fort Extraction'!$C$2:$C$944, P$3, 'Country-Vehicle-Fort Extraction'!$D$2:$D$944, "All",  'Country-Vehicle-Fort Extraction'!$E$2:$E$944, $A8, 'Country-Vehicle-Fort Extraction'!$J$2:$J$944, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="Q8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -6998,7 +7006,7 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>10</v>
@@ -7036,13 +7044,13 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
         <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
@@ -7065,19 +7073,19 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
         <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="I3" t="s">
         <v>47</v>
@@ -7094,13 +7102,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
         <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
@@ -7115,7 +7123,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -7126,19 +7134,19 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
         <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F5" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
@@ -7147,7 +7155,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -7158,13 +7166,13 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D6" t="s">
         <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F6" t="s">
         <v>29</v>
@@ -7179,7 +7187,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -7190,19 +7198,19 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D7" t="s">
         <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="I7" t="s">
         <v>47</v>
@@ -7211,7 +7219,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -7222,13 +7230,13 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
@@ -7243,7 +7251,7 @@
         <v>0.61875637104994907</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -7254,13 +7262,13 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
         <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -7284,13 +7292,13 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
         <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -7314,13 +7322,13 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
         <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -7344,13 +7352,13 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
         <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
@@ -7374,13 +7382,13 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
         <v>41</v>
       </c>
       <c r="E13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -7404,19 +7412,19 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F14" t="s">
+        <v>97</v>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="I14" t="s">
         <v>47</v>
@@ -7425,7 +7433,7 @@
         <v>420</v>
       </c>
       <c r="L14" s="32" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -7436,13 +7444,13 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
         <v>27</v>
       </c>
       <c r="E15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
@@ -7457,7 +7465,7 @@
         <v>0</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -7468,19 +7476,19 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F16" t="s">
+        <v>97</v>
+      </c>
+      <c r="G16" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="I16" t="s">
         <v>47</v>
@@ -7498,28 +7506,28 @@
         <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
         <v>27</v>
       </c>
       <c r="E17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F17" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" t="s">
         <v>98</v>
       </c>
-      <c r="G17" t="s">
-        <v>99</v>
-      </c>
       <c r="I17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J17">
         <v>42.5</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -7530,28 +7538,28 @@
         <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
         <v>27</v>
       </c>
       <c r="E18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F18" t="s">
+        <v>97</v>
+      </c>
+      <c r="G18" t="s">
         <v>98</v>
       </c>
-      <c r="G18" t="s">
-        <v>99</v>
-      </c>
       <c r="I18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J18">
         <v>0.125</v>
       </c>
       <c r="L18" s="32" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
@@ -7562,13 +7570,13 @@
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D19" t="s">
         <v>27</v>
       </c>
       <c r="E19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -7583,7 +7591,7 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
@@ -7594,13 +7602,13 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D20" t="s">
         <v>27</v>
       </c>
       <c r="E20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
         <v>29</v>
@@ -7615,7 +7623,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
@@ -7626,13 +7634,13 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D21" t="s">
         <v>27</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F21" t="s">
         <v>29</v>
@@ -7644,7 +7652,7 @@
         <v>0.8</v>
       </c>
       <c r="L21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -7655,13 +7663,13 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D22" t="s">
         <v>27</v>
       </c>
       <c r="E22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F22" t="s">
         <v>29</v>
@@ -7673,7 +7681,7 @@
         <v>0.8</v>
       </c>
       <c r="L22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
@@ -7684,13 +7692,13 @@
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
         <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F23" t="s">
         <v>29</v>
@@ -7702,7 +7710,7 @@
         <v>0.8</v>
       </c>
       <c r="L23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
@@ -7713,13 +7721,13 @@
         <v>7</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D24" t="s">
         <v>27</v>
       </c>
       <c r="E24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F24" t="s">
         <v>29</v>
@@ -7731,7 +7739,7 @@
         <v>0.8</v>
       </c>
       <c r="L24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
@@ -7742,13 +7750,13 @@
         <v>7</v>
       </c>
       <c r="C25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
       </c>
       <c r="E25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F25" t="s">
         <v>29</v>
@@ -7760,7 +7768,7 @@
         <v>0.8</v>
       </c>
       <c r="L25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -7860,30 +7868,30 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" t="s">
         <v>110</v>
       </c>
-      <c r="B4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>111</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" t="s">
         <v>112</v>
-      </c>
-      <c r="F4" t="s">
-        <v>111</v>
-      </c>
-      <c r="G4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B5" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$2:$A$980, B$1,  'Country Extraction'!$B$2:$B$980, "All",  'Country Extraction'!$C$2:$C$980, $A5) = 0, "Missing", "Complete")</f>
@@ -7912,7 +7920,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B6" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$2:$A$980, B$1,  'Country Extraction'!$B$2:$B$980, "All",  'Country Extraction'!$C$2:$C$980, $A6) = 0, "Missing", "Complete")</f>
@@ -7941,226 +7949,226 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E7" t="s">
         <v>111</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G7" t="s">
         <v>112</v>
-      </c>
-      <c r="F7" t="s">
-        <v>111</v>
-      </c>
-      <c r="G7" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
         <v>111</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G8" t="s">
         <v>112</v>
-      </c>
-      <c r="F8" t="s">
-        <v>111</v>
-      </c>
-      <c r="G8" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H9" t="s">
         <v>118</v>
-      </c>
-      <c r="B9" t="s">
-        <v>94</v>
-      </c>
-      <c r="C9" t="s">
-        <v>94</v>
-      </c>
-      <c r="D9" t="s">
-        <v>111</v>
-      </c>
-      <c r="E9" t="s">
-        <v>112</v>
-      </c>
-      <c r="F9" t="s">
-        <v>111</v>
-      </c>
-      <c r="G9" t="s">
-        <v>113</v>
-      </c>
-      <c r="H9" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E10" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A10, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G10" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, H$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A10, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E11" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A11, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" t="s">
         <v>111</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G12" t="s">
         <v>112</v>
-      </c>
-      <c r="F12" t="s">
-        <v>111</v>
-      </c>
-      <c r="G12" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F13" t="s">
+        <v>110</v>
+      </c>
+      <c r="G13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" t="s">
         <v>125</v>
-      </c>
-      <c r="B13" t="s">
-        <v>94</v>
-      </c>
-      <c r="C13" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" t="s">
-        <v>111</v>
-      </c>
-      <c r="E13" t="s">
-        <v>112</v>
-      </c>
-      <c r="F13" t="s">
-        <v>111</v>
-      </c>
-      <c r="G13" t="s">
-        <v>113</v>
-      </c>
-      <c r="H13" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" t="s">
+        <v>111</v>
+      </c>
+      <c r="F14" t="s">
+        <v>110</v>
+      </c>
+      <c r="G14" t="s">
+        <v>112</v>
+      </c>
+      <c r="H14" t="s">
         <v>127</v>
-      </c>
-      <c r="B14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C14" t="s">
-        <v>94</v>
-      </c>
-      <c r="D14" t="s">
-        <v>111</v>
-      </c>
-      <c r="E14" t="s">
-        <v>112</v>
-      </c>
-      <c r="F14" t="s">
-        <v>111</v>
-      </c>
-      <c r="G14" t="s">
-        <v>113</v>
-      </c>
-      <c r="H14" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, D$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="D15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, F$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="F15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G15" t="str">
         <f>IF(COUNTIFS('Country Extraction'!$A$1:$A$995, H$1, 'Country Extraction'!$B$1:$B$995, "&lt;&gt;All", 'Country Extraction'!$C$1:$C$995, $A15, 'Country Extraction'!$H$1:$H$995, "&lt;&gt;") &lt; 5, "Missing", "Complete")</f>
@@ -8231,19 +8239,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="E2" t="s">
         <v>131</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
+        <v>131</v>
+      </c>
+      <c r="J2" s="11" t="s">
         <v>132</v>
-      </c>
-      <c r="G2" t="s">
-        <v>132</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -8254,16 +8262,16 @@
         <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" t="s">
         <v>131</v>
       </c>
-      <c r="E3" t="s">
-        <v>132</v>
-      </c>
       <c r="G3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -8274,13 +8282,13 @@
         <v>38</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" t="s">
         <v>131</v>
       </c>
-      <c r="E4" t="s">
-        <v>132</v>
-      </c>
       <c r="G4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -8291,13 +8299,13 @@
         <v>39</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" t="s">
         <v>131</v>
       </c>
-      <c r="E5" t="s">
-        <v>132</v>
-      </c>
       <c r="G5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -8308,13 +8316,13 @@
         <v>40</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E6" t="s">
         <v>131</v>
       </c>
-      <c r="E6" t="s">
-        <v>132</v>
-      </c>
       <c r="G6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -8325,115 +8333,115 @@
         <v>41</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" t="s">
         <v>131</v>
       </c>
-      <c r="E7" t="s">
-        <v>132</v>
-      </c>
       <c r="G7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="E8" t="s">
         <v>131</v>
       </c>
-      <c r="E8" t="s">
-        <v>132</v>
-      </c>
       <c r="G8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" t="s">
         <v>131</v>
       </c>
-      <c r="E9" t="s">
-        <v>132</v>
-      </c>
       <c r="G9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" t="s">
         <v>131</v>
       </c>
-      <c r="E10" t="s">
-        <v>132</v>
-      </c>
       <c r="G10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E11" t="s">
         <v>131</v>
       </c>
-      <c r="E11" t="s">
-        <v>132</v>
-      </c>
       <c r="G11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B12" t="s">
         <v>40</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E12" t="s">
         <v>131</v>
       </c>
-      <c r="E12" t="s">
-        <v>132</v>
-      </c>
       <c r="G12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B13" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" t="s">
         <v>131</v>
       </c>
-      <c r="E13" t="s">
-        <v>132</v>
-      </c>
       <c r="G13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -8441,16 +8449,16 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="E14" t="s">
         <v>131</v>
       </c>
-      <c r="E14" t="s">
-        <v>132</v>
-      </c>
       <c r="G14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -8461,13 +8469,13 @@
         <v>37</v>
       </c>
       <c r="C15" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" t="s">
         <v>131</v>
       </c>
-      <c r="E15" t="s">
-        <v>132</v>
-      </c>
       <c r="G15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -8478,13 +8486,13 @@
         <v>38</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E16" t="s">
         <v>131</v>
       </c>
-      <c r="E16" t="s">
-        <v>132</v>
-      </c>
       <c r="G16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -8495,13 +8503,13 @@
         <v>39</v>
       </c>
       <c r="C17" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E17" t="s">
         <v>131</v>
       </c>
-      <c r="E17" t="s">
-        <v>132</v>
-      </c>
       <c r="G17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -8512,13 +8520,13 @@
         <v>40</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E18" t="s">
         <v>131</v>
       </c>
-      <c r="E18" t="s">
-        <v>132</v>
-      </c>
       <c r="G18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -8529,13 +8537,13 @@
         <v>41</v>
       </c>
       <c r="C19" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E19" t="s">
         <v>131</v>
       </c>
-      <c r="E19" t="s">
-        <v>132</v>
-      </c>
       <c r="G19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.4">
@@ -8543,19 +8551,19 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C20" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="G20" t="s">
+        <v>131</v>
+      </c>
+      <c r="J20" s="11" t="s">
         <v>137</v>
-      </c>
-      <c r="G20" t="s">
-        <v>132</v>
-      </c>
-      <c r="J20" s="11" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -8566,16 +8574,16 @@
         <v>37</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E21" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -8586,13 +8594,13 @@
         <v>38</v>
       </c>
       <c r="C22" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E22" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G22" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -8603,13 +8611,13 @@
         <v>39</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -8620,13 +8628,13 @@
         <v>40</v>
       </c>
       <c r="C24" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E24" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G24" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -8637,115 +8645,115 @@
         <v>41</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E25" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E25" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" t="s">
+        <v>129</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B26" t="s">
-        <v>130</v>
-      </c>
-      <c r="C26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E26" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G26" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B27" t="s">
         <v>37</v>
       </c>
       <c r="C27" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E27" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G27" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E28" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
       </c>
       <c r="C29" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E29" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
       </c>
       <c r="C30" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E30" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E30" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B31" t="s">
         <v>41</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E31" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
@@ -8753,16 +8761,16 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E32" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G32" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -8773,13 +8781,13 @@
         <v>37</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E33" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G33" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -8790,13 +8798,13 @@
         <v>38</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E34" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G34" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -8807,13 +8815,13 @@
         <v>39</v>
       </c>
       <c r="C35" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E35" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G35" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -8824,13 +8832,13 @@
         <v>40</v>
       </c>
       <c r="C36" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E36" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E36" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -8841,13 +8849,13 @@
         <v>41</v>
       </c>
       <c r="C37" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E37" s="8" t="s">
-        <v>137</v>
-      </c>
       <c r="G37" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -8855,13 +8863,13 @@
         <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C38" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="G38" s="9" t="s">
         <v>139</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -8872,10 +8880,10 @@
         <v>37</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -8886,10 +8894,10 @@
         <v>38</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -8900,10 +8908,10 @@
         <v>39</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
@@ -8914,10 +8922,10 @@
         <v>40</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -8928,94 +8936,94 @@
         <v>41</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B44" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B45" t="s">
         <v>37</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B46" t="s">
         <v>38</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B47" t="s">
         <v>39</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B48" t="s">
         <v>40</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B49" t="s">
         <v>41</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
@@ -9023,13 +9031,13 @@
         <v>3</v>
       </c>
       <c r="B50" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
@@ -9040,10 +9048,10 @@
         <v>37</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G51" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
@@ -9054,10 +9062,10 @@
         <v>38</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G52" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
@@ -9068,10 +9076,10 @@
         <v>39</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G53" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -9082,10 +9090,10 @@
         <v>40</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G54" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
@@ -9096,10 +9104,10 @@
         <v>41</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G55" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
@@ -9107,13 +9115,13 @@
         <v>1</v>
       </c>
       <c r="B56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C56" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G56" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -9124,10 +9132,10 @@
         <v>37</v>
       </c>
       <c r="C57" t="s">
+        <v>145</v>
+      </c>
+      <c r="J57" s="13" t="s">
         <v>146</v>
-      </c>
-      <c r="J57" s="13" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.4">
@@ -9138,10 +9146,10 @@
         <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.4">
@@ -9152,7 +9160,7 @@
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J59" s="12"/>
     </row>
@@ -9164,7 +9172,7 @@
         <v>40</v>
       </c>
       <c r="C60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
@@ -9175,76 +9183,76 @@
         <v>41</v>
       </c>
       <c r="C61" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B62" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B63" t="s">
         <v>37</v>
       </c>
       <c r="C63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B64" t="s">
         <v>38</v>
       </c>
       <c r="C64" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B65" t="s">
         <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B66" t="s">
         <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B67" t="s">
         <v>41</v>
       </c>
       <c r="C67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
@@ -9252,13 +9260,13 @@
         <v>3</v>
       </c>
       <c r="B68" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C68" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
@@ -9269,7 +9277,7 @@
         <v>37</v>
       </c>
       <c r="C69" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
@@ -9280,7 +9288,7 @@
         <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
@@ -9291,7 +9299,7 @@
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
@@ -9302,7 +9310,7 @@
         <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
@@ -9313,7 +9321,7 @@
         <v>41</v>
       </c>
       <c r="C73" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="29.5" x14ac:dyDescent="0.4">
@@ -9321,36 +9329,36 @@
         <v>1</v>
       </c>
       <c r="B74" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C74" t="s">
+        <v>148</v>
+      </c>
+      <c r="D74" t="s">
         <v>149</v>
       </c>
-      <c r="D74" t="s">
+      <c r="G74" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="G74" s="12" t="s">
+      <c r="J74" s="14" t="s">
         <v>151</v>
-      </c>
-      <c r="J74" s="14" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B75" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C75" t="s">
+        <v>148</v>
+      </c>
+      <c r="D75" t="s">
         <v>149</v>
       </c>
-      <c r="D75" t="s">
-        <v>150</v>
-      </c>
       <c r="J75" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -9358,13 +9366,13 @@
         <v>3</v>
       </c>
       <c r="B76" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C76" t="s">
+        <v>148</v>
+      </c>
+      <c r="D76" t="s">
         <v>149</v>
-      </c>
-      <c r="D76" t="s">
-        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -9440,10 +9448,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C3" t="str">
         <f>IF(COUNTIFS('Vehicle Extraction'!$A$2:$A$904, C$1,  'Vehicle Extraction'!$B$2:$B$904, $A3) = 0, "Missing", "Complete")</f>
@@ -9456,10 +9464,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C4" t="str">
         <f>IF(COUNTIFS('Vehicle Extraction'!$A$2:$A$904, C$1,  'Vehicle Extraction'!$B$2:$B$904, $A4) = 0, "Missing", "Complete")</f>
@@ -9528,28 +9536,28 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" t="s">
         <v>156</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>157</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="G2" s="26">
         <v>3.25</v>
       </c>
       <c r="H2" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -9557,28 +9565,28 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" t="s">
         <v>156</v>
-      </c>
-      <c r="D3" t="s">
-        <v>157</v>
       </c>
       <c r="E3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G3">
         <v>4.4000000000000004</v>
       </c>
       <c r="H3" t="s">
+        <v>162</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>163</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -9586,28 +9594,28 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D4" t="s">
         <v>156</v>
-      </c>
-      <c r="D4" t="s">
-        <v>157</v>
       </c>
       <c r="E4">
         <v>2012</v>
       </c>
       <c r="F4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G4">
         <v>4.2</v>
       </c>
       <c r="H4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -9615,28 +9623,28 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C5" t="s">
         <v>155</v>
       </c>
-      <c r="C5" t="s">
-        <v>156</v>
-      </c>
       <c r="D5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E5">
         <v>2013</v>
       </c>
       <c r="F5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G5">
         <v>1.67</v>
       </c>
       <c r="H5" t="s">
+        <v>169</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>170</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -9644,28 +9652,28 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C6" t="s">
         <v>155</v>
       </c>
-      <c r="C6" t="s">
-        <v>156</v>
-      </c>
       <c r="D6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E6">
         <v>2013</v>
       </c>
       <c r="F6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G6">
         <v>1.67</v>
       </c>
       <c r="H6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>170</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -9737,7 +9745,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -9750,59 +9758,59 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="C3" s="26" t="s">
         <v>174</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>175</v>
       </c>
       <c r="D3" s="26">
         <v>2018</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3" s="26">
         <v>4.3</v>
       </c>
       <c r="G3" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="H3" s="24" t="s">
         <v>177</v>
-      </c>
-      <c r="H3" s="24" t="s">
-        <v>178</v>
       </c>
       <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="B4" s="26" t="s">
         <v>179</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="C4" s="26" t="s">
         <v>180</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>181</v>
       </c>
       <c r="D4" s="26">
         <v>2015</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F4" s="26">
         <v>6</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
@@ -9815,18 +9823,18 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="26" t="s">
         <v>185</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>186</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
       <c r="E6" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="F6" s="26" t="s">
         <v>187</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>188</v>
       </c>
       <c r="G6" s="26"/>
       <c r="H6" s="23"/>
@@ -9834,18 +9842,18 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="26" t="s">
         <v>185</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>186</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
       <c r="E7" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="F7" s="26" t="s">
         <v>189</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>190</v>
       </c>
       <c r="G7" s="26"/>
       <c r="H7" s="23"/>
@@ -9853,22 +9861,22 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="26" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
       <c r="E8" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" s="26" t="s">
         <v>192</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>193</v>
       </c>
       <c r="G8" s="26"/>
       <c r="H8" s="23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I8" s="23"/>
     </row>

</xml_diff>

<commit_message>
Correct issues with wealth disaggregation of consumption data in Nigeria
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/Data Extraction Sheet.xlsx
+++ b/0100_data_prep/extraction/Data Extraction Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30431"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/04_Concept_Model_Development/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6519260-0061-43D4-999E-ACB54C4C2F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{98998835-291D-42E1-972A-CDC08A515183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Country-Vehicle Progress" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2027" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1857" uniqueCount="229">
   <si>
     <t>Country</t>
   </si>
@@ -910,7 +910,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -962,6 +962,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1380,41 +1383,41 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="33"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="2" spans="1:9" ht="15">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33" t="s">
+      <c r="C2" s="34"/>
+      <c r="D2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33" t="s">
+      <c r="E2" s="34"/>
+      <c r="F2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33" t="s">
+      <c r="G2" s="34"/>
+      <c r="H2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="33"/>
+      <c r="I2" s="34"/>
     </row>
     <row r="3" spans="1:9" ht="15">
       <c r="A3" s="3" t="s">
@@ -1461,27 +1464,27 @@
         <v>12</v>
       </c>
       <c r="B5" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A5, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A5, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="C5" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$1009, $A5, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$989, $A5, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="D5" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A5, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A5, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="E5" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A5, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A5, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="F5" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A5, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A5, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="G5" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A5, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A5, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="H5" t="s">
@@ -1496,27 +1499,27 @@
         <v>14</v>
       </c>
       <c r="B6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A6, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A6, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="C6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$1009, $A6, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$989, $A6, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="D6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A6, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A6, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="E6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A6, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A6, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="F6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A6, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A6, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="G6" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A6, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A6, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="H6" t="s">
@@ -1531,27 +1534,27 @@
         <v>15</v>
       </c>
       <c r="B7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A7, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A7, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="C7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$1009, $A7, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$989, $A7, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="D7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A7, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A7, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="E7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A7, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A7, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="F7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A7, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A7, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="G7" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A7, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A7, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="H7" t="s">
@@ -1566,27 +1569,27 @@
         <v>16</v>
       </c>
       <c r="B8" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A8, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A8, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="C8" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$1009, $A8, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$989, $A8, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="D8" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A8, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A8, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="E8" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A8, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A8, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="F8" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A8, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A8, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="G8" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A8, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A8, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="H8" t="s">
@@ -1601,31 +1604,31 @@
         <v>17</v>
       </c>
       <c r="B9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="C9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, B$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, B$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, B$1,  'Country-Vehicle Extraction'!$B$2:$B$989, B$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!E$2:E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="D9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="E9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, D$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, D$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="F9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Missing</v>
       </c>
       <c r="G9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, D$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, F$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, D$1,  'Country-Vehicle Extraction'!$B$2:$B$989, F$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "&lt;&gt;All",  'Country-Vehicle Extraction'!$E$2:$E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="H9" t="str">
-        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$1009, H$1,  'Country-Vehicle Extraction'!$B$2:$B$1009, H$2,  'Country-Vehicle Extraction'!$C$2:$C$1009, "Total",  'Country-Vehicle Extraction'!$E$2:$E$1009, $A9, 'Country-Vehicle Extraction'!$J$2:$J$1009, "&lt;&gt;") = 0, "Missing", "Complete")</f>
+        <f>IF(COUNTIFS('Country-Vehicle Extraction'!$A$2:$A$989, H$1,  'Country-Vehicle Extraction'!$B$2:$B$989, H$2,  'Country-Vehicle Extraction'!$C$2:$C$989, "Total",  'Country-Vehicle Extraction'!$E$2:$E$989, $A9, 'Country-Vehicle Extraction'!$J$2:$J$989, "&lt;&gt;") = 0, "Missing", "Complete")</f>
         <v>Complete</v>
       </c>
       <c r="I9" t="s">
@@ -1668,50 +1671,50 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="33"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="2" spans="1:9" ht="15">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33" t="s">
+      <c r="C2" s="34"/>
+      <c r="D2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33" t="s">
+      <c r="E2" s="34"/>
+      <c r="F2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33" t="s">
+      <c r="G2" s="34"/>
+      <c r="H2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="33"/>
+      <c r="I2" s="34"/>
     </row>
     <row r="3" spans="1:9" ht="15">
       <c r="A3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="34"/>
       <c r="D3" s="28" t="s">
         <v>90</v>
       </c>
@@ -2805,7 +2808,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7501F0-08E1-4A63-A382-F6741C91E79A}">
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:M102"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -2892,7 +2895,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" ht="29.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2920,7 +2923,7 @@
       <c r="J3" s="5">
         <v>7.1</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="5" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4375,16 +4378,16 @@
         <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D46" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E46" t="s">
         <v>16</v>
       </c>
       <c r="F46" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G46" t="s">
         <v>35</v>
@@ -4396,16 +4399,11 @@
         <v>49</v>
       </c>
       <c r="J46">
-        <v>8.4</v>
-      </c>
-      <c r="K46" t="s">
-        <v>62</v>
-      </c>
-      <c r="L46">
-        <v>0.3</v>
+        <f>(5.5-2.5)/1.35</f>
+        <v>2.2222222222222219</v>
       </c>
       <c r="M46" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -4416,16 +4414,16 @@
         <v>6</v>
       </c>
       <c r="C47" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D47" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E47" t="s">
         <v>16</v>
       </c>
       <c r="F47" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G47" t="s">
         <v>35</v>
@@ -4436,17 +4434,12 @@
       <c r="I47" t="s">
         <v>49</v>
       </c>
-      <c r="J47" s="18">
-        <v>8</v>
-      </c>
-      <c r="K47" t="s">
-        <v>63</v>
-      </c>
-      <c r="L47">
-        <v>0.3</v>
+      <c r="J47">
+        <f>(5.4-2.4)/1.35</f>
+        <v>2.2222222222222223</v>
       </c>
       <c r="M47" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -4457,16 +4450,16 @@
         <v>6</v>
       </c>
       <c r="C48" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D48" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E48" t="s">
         <v>16</v>
       </c>
       <c r="F48" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G48" t="s">
         <v>35</v>
@@ -4478,16 +4471,14 @@
         <v>49</v>
       </c>
       <c r="J48">
-        <v>5.9</v>
-      </c>
-      <c r="K48" t="s">
-        <v>65</v>
-      </c>
-      <c r="L48">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13">
+        <f>(5.6-2.5)/1.35</f>
+        <v>2.2962962962962958</v>
+      </c>
+      <c r="M48" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" ht="144.75">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -4495,19 +4486,19 @@
         <v>6</v>
       </c>
       <c r="C49" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D49" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E49" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F49" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G49" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H49">
         <v>2021</v>
@@ -4515,14 +4506,13 @@
       <c r="I49" t="s">
         <v>49</v>
       </c>
-      <c r="J49">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="K49" t="s">
-        <v>67</v>
-      </c>
-      <c r="L49">
-        <v>0.3</v>
+      <c r="J49" s="21">
+        <v>0.97961264016309901</v>
+      </c>
+      <c r="K49" s="17"/>
+      <c r="L49" s="17"/>
+      <c r="M49" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -4533,19 +4523,19 @@
         <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D50" t="s">
         <v>27</v>
       </c>
       <c r="E50" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G50" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H50">
         <v>2021</v>
@@ -4553,14 +4543,8 @@
       <c r="I50" t="s">
         <v>49</v>
       </c>
-      <c r="J50">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="K50" t="s">
-        <v>68</v>
-      </c>
-      <c r="L50">
-        <v>0.3</v>
+      <c r="J50" s="17">
+        <v>0.96573208722741399</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -4571,19 +4555,19 @@
         <v>6</v>
       </c>
       <c r="C51" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D51" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E51" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F51" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G51" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H51">
         <v>2021</v>
@@ -4591,12 +4575,8 @@
       <c r="I51" t="s">
         <v>49</v>
       </c>
-      <c r="J51">
-        <f>(5.5-2.5)/1.35</f>
-        <v>2.2222222222222219</v>
-      </c>
-      <c r="M51" t="s">
-        <v>79</v>
+      <c r="J51" s="7">
+        <v>0.9785932721712538</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -4607,19 +4587,19 @@
         <v>6</v>
       </c>
       <c r="C52" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D52" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E52" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F52" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G52" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H52">
         <v>2021</v>
@@ -4627,12 +4607,8 @@
       <c r="I52" t="s">
         <v>49</v>
       </c>
-      <c r="J52">
-        <f>(5.4-2.4)/1.35</f>
-        <v>2.2222222222222223</v>
-      </c>
-      <c r="M52" t="s">
-        <v>79</v>
+      <c r="J52" s="20">
+        <v>0.98084677419354838</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -4643,19 +4619,19 @@
         <v>6</v>
       </c>
       <c r="C53" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D53" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E53" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F53" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G53" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H53">
         <v>2021</v>
@@ -4663,12 +4639,8 @@
       <c r="I53" t="s">
         <v>49</v>
       </c>
-      <c r="J53">
-        <f>(5.6-2.5)/1.35</f>
-        <v>2.2962962962962958</v>
-      </c>
-      <c r="M53" t="s">
-        <v>79</v>
+      <c r="J53" s="7">
+        <v>0.98884381338742389</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -4679,19 +4651,19 @@
         <v>6</v>
       </c>
       <c r="C54" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D54" t="s">
         <v>27</v>
       </c>
       <c r="E54" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G54" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H54">
         <v>2021</v>
@@ -4699,95 +4671,95 @@
       <c r="I54" t="s">
         <v>49</v>
       </c>
-      <c r="J54">
-        <v>3.6296296296296298</v>
-      </c>
-      <c r="M54" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13">
+      <c r="J54" s="20">
+        <v>0.98377281947261663</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" ht="57.75">
       <c r="A55" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C55" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D55" t="s">
         <v>27</v>
       </c>
       <c r="E55" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F55" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G55" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H55">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="I55" t="s">
-        <v>49</v>
-      </c>
-      <c r="J55">
-        <v>3.1111111111111112</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13">
+        <v>47</v>
+      </c>
+      <c r="J55" s="21">
+        <v>0</v>
+      </c>
+      <c r="M55" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" ht="15">
       <c r="A56" t="s">
         <v>2</v>
       </c>
       <c r="B56" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C56" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D56" t="s">
         <v>27</v>
       </c>
       <c r="E56" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F56" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G56" t="s">
-        <v>35</v>
-      </c>
-      <c r="H56">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I56" t="s">
-        <v>49</v>
-      </c>
-      <c r="J56" s="18">
-        <v>2.9629629629629624</v>
-      </c>
-    </row>
-    <row r="57" spans="1:13">
+        <v>47</v>
+      </c>
+      <c r="J56" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="M56" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" ht="43.5">
       <c r="A57" t="s">
         <v>2</v>
       </c>
       <c r="B57" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C57" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D57" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E57" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F57" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G57" t="s">
         <v>35</v>
@@ -4799,27 +4771,31 @@
         <v>49</v>
       </c>
       <c r="J57">
-        <v>2.4444444444444446</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13">
+        <f>61.2*J63</f>
+        <v>32.803200000000004</v>
+      </c>
+      <c r="M57" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" ht="43.5">
       <c r="A58" t="s">
         <v>2</v>
       </c>
       <c r="B58" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C58" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D58" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E58" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F58" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G58" t="s">
         <v>35</v>
@@ -4831,30 +4807,34 @@
         <v>49</v>
       </c>
       <c r="J58">
-        <v>1.7037037037037035</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13">
+        <f>34.2*J64</f>
+        <v>11.491200000000001</v>
+      </c>
+      <c r="M58" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" ht="43.5">
       <c r="A59" t="s">
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C59" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D59" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E59" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F59" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G59" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H59">
         <v>2021</v>
@@ -4862,36 +4842,35 @@
       <c r="I59" t="s">
         <v>49</v>
       </c>
-      <c r="J59" s="21">
-        <v>0.9796126401630989</v>
-      </c>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
-      <c r="M59" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13">
+      <c r="J59">
+        <f>52.4*J65</f>
+        <v>23.475200000000001</v>
+      </c>
+      <c r="M59" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" ht="43.5">
       <c r="A60" t="s">
         <v>2</v>
       </c>
       <c r="B60" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C60" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D60" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E60" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F60" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G60" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H60">
         <v>2021</v>
@@ -4899,31 +4878,35 @@
       <c r="I60" t="s">
         <v>49</v>
       </c>
-      <c r="J60" s="17">
-        <v>0.96573208722741399</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13">
+      <c r="J60">
+        <f>60.7*J66</f>
+        <v>33.142200000000003</v>
+      </c>
+      <c r="M60" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" ht="43.5">
       <c r="A61" t="s">
         <v>2</v>
       </c>
       <c r="B61" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C61" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D61" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E61" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F61" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G61" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H61">
         <v>2021</v>
@@ -4931,31 +4914,35 @@
       <c r="I61" t="s">
         <v>49</v>
       </c>
-      <c r="J61" s="7">
-        <v>0.9785932721712538</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13">
+      <c r="J61">
+        <f>73.7*J67</f>
+        <v>46.652100000000004</v>
+      </c>
+      <c r="M61" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" ht="43.5">
       <c r="A62" t="s">
         <v>2</v>
       </c>
       <c r="B62" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C62" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D62" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E62" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F62" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G62" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H62">
         <v>2021</v>
@@ -4963,25 +4950,29 @@
       <c r="I62" t="s">
         <v>49</v>
       </c>
-      <c r="J62" s="20">
-        <v>0.98084677419354838</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13">
+      <c r="J62">
+        <f>79.5*J68</f>
+        <v>53.742000000000004</v>
+      </c>
+      <c r="M62" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" ht="29.25">
       <c r="A63" t="s">
         <v>2</v>
       </c>
       <c r="B63" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C63" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D63" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E63" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F63" t="s">
         <v>29</v>
@@ -4989,14 +4980,14 @@
       <c r="G63" t="s">
         <v>30</v>
       </c>
-      <c r="H63">
-        <v>2021</v>
-      </c>
       <c r="I63" t="s">
-        <v>49</v>
-      </c>
-      <c r="J63" s="7">
-        <v>0.98884381338742389</v>
+        <v>84</v>
+      </c>
+      <c r="J63" s="21">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="M63" s="5" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -5004,16 +4995,16 @@
         <v>2</v>
       </c>
       <c r="B64" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D64" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E64" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F64" t="s">
         <v>29</v>
@@ -5021,31 +5012,28 @@
       <c r="G64" t="s">
         <v>30</v>
       </c>
-      <c r="H64">
-        <v>2021</v>
-      </c>
       <c r="I64" t="s">
-        <v>49</v>
-      </c>
-      <c r="J64" s="20">
-        <v>0.98377281947261663</v>
-      </c>
-    </row>
-    <row r="65" spans="1:13" ht="57.75">
+        <v>84</v>
+      </c>
+      <c r="J64" s="21">
+        <v>0.33600000000000002</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13">
       <c r="A65" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B65" t="s">
         <v>7</v>
       </c>
       <c r="C65" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D65" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E65" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F65" t="s">
         <v>29</v>
@@ -5053,20 +5041,14 @@
       <c r="G65" t="s">
         <v>30</v>
       </c>
-      <c r="H65">
-        <v>2024</v>
-      </c>
       <c r="I65" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="J65" s="21">
-        <v>0</v>
-      </c>
-      <c r="M65" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" ht="15">
+        <v>0.44800000000000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -5074,13 +5056,13 @@
         <v>7</v>
       </c>
       <c r="C66" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D66" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E66" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F66" t="s">
         <v>29</v>
@@ -5089,16 +5071,13 @@
         <v>30</v>
       </c>
       <c r="I66" t="s">
-        <v>47</v>
-      </c>
-      <c r="J66" s="7">
-        <v>0.3</v>
-      </c>
-      <c r="M66" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="67" spans="1:13" ht="43.5">
+        <v>84</v>
+      </c>
+      <c r="J66" s="21">
+        <v>0.54600000000000004</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13">
       <c r="A67" t="s">
         <v>2</v>
       </c>
@@ -5106,35 +5085,28 @@
         <v>7</v>
       </c>
       <c r="C67" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D67" t="s">
         <v>28</v>
       </c>
       <c r="E67" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F67" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G67" t="s">
-        <v>35</v>
-      </c>
-      <c r="H67">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I67" t="s">
-        <v>49</v>
-      </c>
-      <c r="J67">
-        <f>61.2*J73</f>
-        <v>32.803200000000004</v>
-      </c>
-      <c r="M67" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="68" spans="1:13" ht="43.5">
+        <v>84</v>
+      </c>
+      <c r="J67" s="21">
+        <v>0.63300000000000001</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13">
       <c r="A68" t="s">
         <v>2</v>
       </c>
@@ -5142,35 +5114,28 @@
         <v>7</v>
       </c>
       <c r="C68" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D68" t="s">
         <v>28</v>
       </c>
       <c r="E68" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F68" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G68" t="s">
-        <v>35</v>
-      </c>
-      <c r="H68">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I68" t="s">
-        <v>49</v>
-      </c>
-      <c r="J68">
-        <f>34.2*J74</f>
-        <v>11.491200000000001</v>
-      </c>
-      <c r="M68" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="69" spans="1:13" ht="43.5">
+        <v>84</v>
+      </c>
+      <c r="J68" s="21">
+        <v>0.67600000000000005</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" ht="29.25">
       <c r="A69" t="s">
         <v>2</v>
       </c>
@@ -5178,7 +5143,7 @@
         <v>7</v>
       </c>
       <c r="C69" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D69" t="s">
         <v>28</v>
@@ -5187,7 +5152,7 @@
         <v>14</v>
       </c>
       <c r="F69" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G69" t="s">
         <v>35</v>
@@ -5199,14 +5164,14 @@
         <v>49</v>
       </c>
       <c r="J69">
-        <f>52.4*J75</f>
-        <v>23.475200000000001</v>
+        <f>(84.6-30.5)/1.35</f>
+        <v>40.074074074074069</v>
       </c>
       <c r="M69" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="70" spans="1:13" ht="43.5">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13">
       <c r="A70" t="s">
         <v>2</v>
       </c>
@@ -5214,7 +5179,7 @@
         <v>7</v>
       </c>
       <c r="C70" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D70" t="s">
         <v>28</v>
@@ -5223,7 +5188,7 @@
         <v>14</v>
       </c>
       <c r="F70" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G70" t="s">
         <v>35</v>
@@ -5235,14 +5200,11 @@
         <v>49</v>
       </c>
       <c r="J70">
-        <f>60.7*J76</f>
-        <v>33.142200000000003</v>
-      </c>
-      <c r="M70" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="71" spans="1:13" ht="43.5">
+        <f>(47.2-13.7)/1.35</f>
+        <v>24.814814814814813</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13">
       <c r="A71" t="s">
         <v>2</v>
       </c>
@@ -5250,7 +5212,7 @@
         <v>7</v>
       </c>
       <c r="C71" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D71" t="s">
         <v>28</v>
@@ -5259,7 +5221,7 @@
         <v>14</v>
       </c>
       <c r="F71" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G71" t="s">
         <v>35</v>
@@ -5271,14 +5233,11 @@
         <v>49</v>
       </c>
       <c r="J71">
-        <f>73.7*J77</f>
-        <v>46.652100000000004</v>
-      </c>
-      <c r="M71" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="72" spans="1:13" ht="43.5">
+        <f>(71.4-26.4)/1.35</f>
+        <v>33.333333333333336</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13">
       <c r="A72" t="s">
         <v>2</v>
       </c>
@@ -5286,7 +5245,7 @@
         <v>7</v>
       </c>
       <c r="C72" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D72" t="s">
         <v>28</v>
@@ -5295,7 +5254,7 @@
         <v>14</v>
       </c>
       <c r="F72" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G72" t="s">
         <v>35</v>
@@ -5307,14 +5266,11 @@
         <v>49</v>
       </c>
       <c r="J72">
-        <f>79.5*J78</f>
-        <v>53.742000000000004</v>
-      </c>
-      <c r="M72" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="73" spans="1:13" ht="29.25">
+        <f>(81.1-33.8)/1.35</f>
+        <v>35.037037037037031</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13">
       <c r="A73" t="s">
         <v>2</v>
       </c>
@@ -5322,28 +5278,29 @@
         <v>7</v>
       </c>
       <c r="C73" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D73" t="s">
         <v>28</v>
       </c>
       <c r="E73" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F73" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G73" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="H73">
+        <v>2021</v>
       </c>
       <c r="I73" t="s">
-        <v>84</v>
-      </c>
-      <c r="J73" s="21">
-        <v>0.53600000000000003</v>
-      </c>
-      <c r="M73" s="5" t="s">
-        <v>85</v>
+        <v>49</v>
+      </c>
+      <c r="J73">
+        <f>(96.3-45.3)/1.35</f>
+        <v>37.777777777777779</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -5354,28 +5311,32 @@
         <v>7</v>
       </c>
       <c r="C74" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D74" t="s">
         <v>28</v>
       </c>
       <c r="E74" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F74" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G74" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="H74">
+        <v>2021</v>
       </c>
       <c r="I74" t="s">
-        <v>84</v>
-      </c>
-      <c r="J74" s="21">
-        <v>0.33600000000000002</v>
-      </c>
-    </row>
-    <row r="75" spans="1:13">
+        <v>49</v>
+      </c>
+      <c r="J74">
+        <f>(103.1-50.4)/1.35</f>
+        <v>39.037037037037031</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" ht="43.5">
       <c r="A75" t="s">
         <v>2</v>
       </c>
@@ -5383,28 +5344,35 @@
         <v>7</v>
       </c>
       <c r="C75" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D75" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E75" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F75" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G75" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="H75">
+        <v>2021</v>
       </c>
       <c r="I75" t="s">
-        <v>84</v>
-      </c>
-      <c r="J75" s="21">
-        <v>0.44800000000000001</v>
-      </c>
-    </row>
-    <row r="76" spans="1:13">
+        <v>49</v>
+      </c>
+      <c r="J75">
+        <f>38.3*J81</f>
+        <v>20.5288</v>
+      </c>
+      <c r="M75" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" ht="43.5">
       <c r="A76" t="s">
         <v>2</v>
       </c>
@@ -5412,28 +5380,35 @@
         <v>7</v>
       </c>
       <c r="C76" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D76" t="s">
         <v>28</v>
       </c>
       <c r="E76" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F76" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G76" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="H76">
+        <v>2021</v>
       </c>
       <c r="I76" t="s">
-        <v>84</v>
-      </c>
-      <c r="J76" s="21">
-        <v>0.54600000000000004</v>
-      </c>
-    </row>
-    <row r="77" spans="1:13">
+        <v>49</v>
+      </c>
+      <c r="J76">
+        <f>35.5*J81</f>
+        <v>19.028000000000002</v>
+      </c>
+      <c r="M76" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" ht="43.5">
       <c r="A77" t="s">
         <v>2</v>
       </c>
@@ -5441,28 +5416,35 @@
         <v>7</v>
       </c>
       <c r="C77" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D77" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="E77" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F77" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G77" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="H77">
+        <v>2021</v>
       </c>
       <c r="I77" t="s">
-        <v>84</v>
-      </c>
-      <c r="J77" s="21">
-        <v>0.63300000000000001</v>
-      </c>
-    </row>
-    <row r="78" spans="1:13">
+        <v>49</v>
+      </c>
+      <c r="J77">
+        <f>41*J81</f>
+        <v>21.976000000000003</v>
+      </c>
+      <c r="M77" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" ht="29.25">
       <c r="A78" t="s">
         <v>2</v>
       </c>
@@ -5470,25 +5452,32 @@
         <v>7</v>
       </c>
       <c r="C78" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D78" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E78" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F78" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="H78">
+        <v>2021</v>
       </c>
       <c r="I78" t="s">
-        <v>84</v>
-      </c>
-      <c r="J78" s="21">
-        <v>0.67600000000000005</v>
+        <v>49</v>
+      </c>
+      <c r="J78">
+        <f>(53.6-19)/1.35</f>
+        <v>25.62962962962963</v>
+      </c>
+      <c r="M78" s="5" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="79" spans="1:13" ht="29.25">
@@ -5505,7 +5494,7 @@
         <v>28</v>
       </c>
       <c r="E79" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F79" t="s">
         <v>42</v>
@@ -5520,14 +5509,14 @@
         <v>49</v>
       </c>
       <c r="J79">
-        <f>(84.6-30.5)/1.35</f>
-        <v>40.074074074074069</v>
+        <f>(49.5-17.1)/1.35</f>
+        <v>23.999999999999996</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="80" spans="1:13">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" ht="29.25">
       <c r="A80" t="s">
         <v>2</v>
       </c>
@@ -5535,13 +5524,13 @@
         <v>7</v>
       </c>
       <c r="C80" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D80" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="E80" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F80" t="s">
         <v>42</v>
@@ -5556,11 +5545,14 @@
         <v>49</v>
       </c>
       <c r="J80">
-        <f>(47.2-13.7)/1.35</f>
-        <v>24.814814814814813</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13">
+        <f>(57.6-20.7)/1.35</f>
+        <v>27.333333333333336</v>
+      </c>
+      <c r="M80" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" ht="29.25">
       <c r="A81" t="s">
         <v>2</v>
       </c>
@@ -5568,29 +5560,28 @@
         <v>7</v>
       </c>
       <c r="C81" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D81" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E81" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F81" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G81" t="s">
-        <v>35</v>
-      </c>
-      <c r="H81">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I81" t="s">
-        <v>49</v>
-      </c>
-      <c r="J81">
-        <f>(71.4-26.4)/1.35</f>
-        <v>33.333333333333336</v>
+        <v>84</v>
+      </c>
+      <c r="J81" s="21">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="M81" s="5" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -5601,29 +5592,25 @@
         <v>7</v>
       </c>
       <c r="C82" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D82" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E82" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F82" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G82" t="s">
-        <v>35</v>
-      </c>
-      <c r="H82">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I82" t="s">
-        <v>49</v>
-      </c>
-      <c r="J82">
-        <f>(81.1-33.8)/1.35</f>
-        <v>35.037037037037031</v>
+        <v>84</v>
+      </c>
+      <c r="J82" s="21">
+        <v>0.33600000000000002</v>
       </c>
     </row>
     <row r="83" spans="1:13">
@@ -5634,29 +5621,25 @@
         <v>7</v>
       </c>
       <c r="C83" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D83" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E83" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F83" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G83" t="s">
-        <v>35</v>
-      </c>
-      <c r="H83">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I83" t="s">
-        <v>49</v>
-      </c>
-      <c r="J83">
-        <f>(96.3-45.3)/1.35</f>
-        <v>37.777777777777779</v>
+        <v>84</v>
+      </c>
+      <c r="J83" s="21">
+        <v>0.44800000000000001</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -5667,32 +5650,28 @@
         <v>7</v>
       </c>
       <c r="C84" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D84" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E84" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F84" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G84" t="s">
-        <v>35</v>
-      </c>
-      <c r="H84">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I84" t="s">
-        <v>49</v>
-      </c>
-      <c r="J84">
-        <f>(103.1-50.4)/1.35</f>
-        <v>39.037037037037031</v>
-      </c>
-    </row>
-    <row r="85" spans="1:13" ht="43.5">
+        <v>84</v>
+      </c>
+      <c r="J84" s="21">
+        <v>0.54600000000000004</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13">
       <c r="A85" t="s">
         <v>2</v>
       </c>
@@ -5700,35 +5679,28 @@
         <v>7</v>
       </c>
       <c r="C85" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D85" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E85" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F85" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G85" t="s">
-        <v>35</v>
-      </c>
-      <c r="H85">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I85" t="s">
-        <v>49</v>
-      </c>
-      <c r="J85">
-        <f>38.3*J101</f>
-        <v>20.5288</v>
-      </c>
-      <c r="M85" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="86" spans="1:13" ht="43.5">
+        <v>84</v>
+      </c>
+      <c r="J85" s="21">
+        <v>0.63300000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13">
       <c r="A86" t="s">
         <v>2</v>
       </c>
@@ -5736,686 +5708,31 @@
         <v>7</v>
       </c>
       <c r="C86" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D86" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E86" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F86" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G86" t="s">
-        <v>35</v>
-      </c>
-      <c r="H86">
-        <v>2021</v>
+        <v>30</v>
       </c>
       <c r="I86" t="s">
-        <v>49</v>
-      </c>
-      <c r="J86">
-        <f>35.5*J101</f>
-        <v>19.028000000000002</v>
-      </c>
-      <c r="M86" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="87" spans="1:13" ht="43.5">
-      <c r="A87" t="s">
-        <v>2</v>
-      </c>
-      <c r="B87" t="s">
-        <v>7</v>
-      </c>
-      <c r="C87" t="s">
-        <v>33</v>
-      </c>
-      <c r="D87" t="s">
-        <v>77</v>
-      </c>
-      <c r="E87" t="s">
-        <v>16</v>
-      </c>
-      <c r="F87" t="s">
-        <v>34</v>
-      </c>
-      <c r="G87" t="s">
-        <v>35</v>
-      </c>
-      <c r="H87">
-        <v>2021</v>
-      </c>
-      <c r="I87" t="s">
-        <v>49</v>
-      </c>
-      <c r="J87">
-        <f>41*J101</f>
-        <v>21.976000000000003</v>
-      </c>
-      <c r="M87" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="88" spans="1:13">
-      <c r="A88" t="s">
-        <v>2</v>
-      </c>
-      <c r="B88" t="s">
-        <v>7</v>
-      </c>
-      <c r="C88" t="s">
-        <v>37</v>
-      </c>
-      <c r="D88" t="s">
-        <v>27</v>
-      </c>
-      <c r="E88" t="s">
-        <v>16</v>
-      </c>
-      <c r="F88" t="s">
-        <v>34</v>
-      </c>
-      <c r="G88" t="s">
-        <v>35</v>
-      </c>
-      <c r="H88">
-        <v>2021</v>
-      </c>
-      <c r="I88" t="s">
-        <v>49</v>
-      </c>
-      <c r="J88">
-        <v>11.491200000000001</v>
-      </c>
-      <c r="M88" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="89" spans="1:13">
-      <c r="A89" t="s">
-        <v>2</v>
-      </c>
-      <c r="B89" t="s">
-        <v>7</v>
-      </c>
-      <c r="C89" t="s">
-        <v>38</v>
-      </c>
-      <c r="D89" t="s">
-        <v>27</v>
-      </c>
-      <c r="E89" t="s">
-        <v>16</v>
-      </c>
-      <c r="F89" t="s">
-        <v>34</v>
-      </c>
-      <c r="G89" t="s">
-        <v>35</v>
-      </c>
-      <c r="H89">
-        <v>2021</v>
-      </c>
-      <c r="I89" t="s">
-        <v>49</v>
-      </c>
-      <c r="J89">
-        <v>23.475200000000001</v>
-      </c>
-    </row>
-    <row r="90" spans="1:13">
-      <c r="A90" t="s">
-        <v>2</v>
-      </c>
-      <c r="B90" t="s">
-        <v>7</v>
-      </c>
-      <c r="C90" t="s">
-        <v>39</v>
-      </c>
-      <c r="D90" t="s">
-        <v>27</v>
-      </c>
-      <c r="E90" t="s">
-        <v>16</v>
-      </c>
-      <c r="F90" t="s">
-        <v>34</v>
-      </c>
-      <c r="G90" t="s">
-        <v>35</v>
-      </c>
-      <c r="H90">
-        <v>2021</v>
-      </c>
-      <c r="I90" t="s">
-        <v>49</v>
-      </c>
-      <c r="J90">
-        <v>33.142200000000003</v>
-      </c>
-    </row>
-    <row r="91" spans="1:13">
-      <c r="A91" t="s">
-        <v>2</v>
-      </c>
-      <c r="B91" t="s">
-        <v>7</v>
-      </c>
-      <c r="C91" t="s">
-        <v>40</v>
-      </c>
-      <c r="D91" t="s">
-        <v>27</v>
-      </c>
-      <c r="E91" t="s">
-        <v>16</v>
-      </c>
-      <c r="F91" t="s">
-        <v>34</v>
-      </c>
-      <c r="G91" t="s">
-        <v>35</v>
-      </c>
-      <c r="H91">
-        <v>2021</v>
-      </c>
-      <c r="I91" t="s">
-        <v>49</v>
-      </c>
-      <c r="J91">
-        <v>46.652100000000004</v>
-      </c>
-    </row>
-    <row r="92" spans="1:13">
-      <c r="A92" t="s">
-        <v>2</v>
-      </c>
-      <c r="B92" t="s">
-        <v>7</v>
-      </c>
-      <c r="C92" t="s">
-        <v>41</v>
-      </c>
-      <c r="D92" t="s">
-        <v>27</v>
-      </c>
-      <c r="E92" t="s">
-        <v>16</v>
-      </c>
-      <c r="F92" t="s">
-        <v>34</v>
-      </c>
-      <c r="G92" t="s">
-        <v>35</v>
-      </c>
-      <c r="H92">
-        <v>2021</v>
-      </c>
-      <c r="I92" t="s">
-        <v>49</v>
-      </c>
-      <c r="J92">
-        <v>53.742000000000004</v>
-      </c>
-    </row>
-    <row r="93" spans="1:13" ht="29.25">
-      <c r="A93" t="s">
-        <v>2</v>
-      </c>
-      <c r="B93" t="s">
-        <v>7</v>
-      </c>
-      <c r="C93" t="s">
-        <v>33</v>
-      </c>
-      <c r="D93" t="s">
-        <v>33</v>
-      </c>
-      <c r="E93" t="s">
-        <v>16</v>
-      </c>
-      <c r="F93" t="s">
-        <v>42</v>
-      </c>
-      <c r="G93" t="s">
-        <v>35</v>
-      </c>
-      <c r="H93">
-        <v>2021</v>
-      </c>
-      <c r="I93" t="s">
-        <v>49</v>
-      </c>
-      <c r="J93">
-        <f>(53.6-19)/1.35</f>
-        <v>25.62962962962963</v>
-      </c>
-      <c r="M93" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" ht="29.25">
-      <c r="A94" t="s">
-        <v>2</v>
-      </c>
-      <c r="B94" t="s">
-        <v>7</v>
-      </c>
-      <c r="C94" t="s">
-        <v>33</v>
-      </c>
-      <c r="D94" t="s">
-        <v>28</v>
-      </c>
-      <c r="E94" t="s">
-        <v>16</v>
-      </c>
-      <c r="F94" t="s">
-        <v>42</v>
-      </c>
-      <c r="G94" t="s">
-        <v>35</v>
-      </c>
-      <c r="H94">
-        <v>2021</v>
-      </c>
-      <c r="I94" t="s">
-        <v>49</v>
-      </c>
-      <c r="J94">
-        <f>(49.5-17.1)/1.35</f>
-        <v>23.999999999999996</v>
-      </c>
-      <c r="M94" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" ht="29.25">
-      <c r="A95" t="s">
-        <v>2</v>
-      </c>
-      <c r="B95" t="s">
-        <v>7</v>
-      </c>
-      <c r="C95" t="s">
-        <v>33</v>
-      </c>
-      <c r="D95" t="s">
-        <v>77</v>
-      </c>
-      <c r="E95" t="s">
-        <v>16</v>
-      </c>
-      <c r="F95" t="s">
-        <v>42</v>
-      </c>
-      <c r="G95" t="s">
-        <v>35</v>
-      </c>
-      <c r="H95">
-        <v>2021</v>
-      </c>
-      <c r="I95" t="s">
-        <v>49</v>
-      </c>
-      <c r="J95">
-        <f>(57.6-20.7)/1.35</f>
-        <v>27.333333333333336</v>
-      </c>
-      <c r="M95" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="96" spans="1:13">
-      <c r="A96" t="s">
-        <v>2</v>
-      </c>
-      <c r="B96" t="s">
-        <v>7</v>
-      </c>
-      <c r="C96" t="s">
-        <v>37</v>
-      </c>
-      <c r="D96" t="s">
-        <v>27</v>
-      </c>
-      <c r="E96" t="s">
-        <v>16</v>
-      </c>
-      <c r="F96" t="s">
-        <v>42</v>
-      </c>
-      <c r="G96" t="s">
-        <v>35</v>
-      </c>
-      <c r="H96">
-        <v>2021</v>
-      </c>
-      <c r="I96" t="s">
-        <v>49</v>
-      </c>
-      <c r="J96">
-        <f>(47.2-13.7)/1.35</f>
-        <v>24.814814814814813</v>
-      </c>
-      <c r="M96" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="97" spans="1:13">
-      <c r="A97" t="s">
-        <v>2</v>
-      </c>
-      <c r="B97" t="s">
-        <v>7</v>
-      </c>
-      <c r="C97" t="s">
-        <v>38</v>
-      </c>
-      <c r="D97" t="s">
-        <v>27</v>
-      </c>
-      <c r="E97" t="s">
-        <v>16</v>
-      </c>
-      <c r="F97" t="s">
-        <v>42</v>
-      </c>
-      <c r="G97" t="s">
-        <v>35</v>
-      </c>
-      <c r="H97">
-        <v>2021</v>
-      </c>
-      <c r="I97" t="s">
-        <v>49</v>
-      </c>
-      <c r="J97">
-        <f>(71.4-26.4)/1.35</f>
-        <v>33.333333333333336</v>
-      </c>
-    </row>
-    <row r="98" spans="1:13">
-      <c r="A98" t="s">
-        <v>2</v>
-      </c>
-      <c r="B98" t="s">
-        <v>7</v>
-      </c>
-      <c r="C98" t="s">
-        <v>39</v>
-      </c>
-      <c r="D98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E98" t="s">
-        <v>16</v>
-      </c>
-      <c r="F98" t="s">
-        <v>42</v>
-      </c>
-      <c r="G98" t="s">
-        <v>35</v>
-      </c>
-      <c r="H98">
-        <v>2021</v>
-      </c>
-      <c r="I98" t="s">
-        <v>49</v>
-      </c>
-      <c r="J98">
-        <f>(81.1-33.8)/1.35</f>
-        <v>35.037037037037031</v>
-      </c>
-    </row>
-    <row r="99" spans="1:13">
-      <c r="A99" t="s">
-        <v>2</v>
-      </c>
-      <c r="B99" t="s">
-        <v>7</v>
-      </c>
-      <c r="C99" t="s">
-        <v>40</v>
-      </c>
-      <c r="D99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E99" t="s">
-        <v>16</v>
-      </c>
-      <c r="F99" t="s">
-        <v>42</v>
-      </c>
-      <c r="G99" t="s">
-        <v>35</v>
-      </c>
-      <c r="H99">
-        <v>2021</v>
-      </c>
-      <c r="I99" t="s">
-        <v>49</v>
-      </c>
-      <c r="J99">
-        <f>(96.3-45.3)/1.35</f>
-        <v>37.777777777777779</v>
-      </c>
-    </row>
-    <row r="100" spans="1:13">
-      <c r="A100" t="s">
-        <v>2</v>
-      </c>
-      <c r="B100" t="s">
-        <v>7</v>
-      </c>
-      <c r="C100" t="s">
-        <v>41</v>
-      </c>
-      <c r="D100" t="s">
-        <v>27</v>
-      </c>
-      <c r="E100" t="s">
-        <v>16</v>
-      </c>
-      <c r="F100" t="s">
-        <v>42</v>
-      </c>
-      <c r="G100" t="s">
-        <v>35</v>
-      </c>
-      <c r="H100">
-        <v>2021</v>
-      </c>
-      <c r="I100" t="s">
-        <v>49</v>
-      </c>
-      <c r="J100">
-        <f>(103.1-50.4)/1.35</f>
-        <v>39.037037037037031</v>
-      </c>
-    </row>
-    <row r="101" spans="1:13" ht="29.25">
-      <c r="A101" t="s">
-        <v>2</v>
-      </c>
-      <c r="B101" t="s">
-        <v>7</v>
-      </c>
-      <c r="C101" t="s">
-        <v>33</v>
-      </c>
-      <c r="D101" t="s">
-        <v>27</v>
-      </c>
-      <c r="E101" t="s">
-        <v>15</v>
-      </c>
-      <c r="F101" t="s">
-        <v>29</v>
-      </c>
-      <c r="G101" t="s">
-        <v>30</v>
-      </c>
-      <c r="I101" t="s">
         <v>84</v>
       </c>
-      <c r="J101" s="21">
-        <v>0.53600000000000003</v>
-      </c>
-      <c r="M101" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="102" spans="1:13">
-      <c r="A102" t="s">
-        <v>2</v>
-      </c>
-      <c r="B102" t="s">
-        <v>7</v>
-      </c>
-      <c r="C102" t="s">
-        <v>37</v>
-      </c>
-      <c r="D102" t="s">
-        <v>27</v>
-      </c>
-      <c r="E102" t="s">
-        <v>15</v>
-      </c>
-      <c r="F102" t="s">
-        <v>29</v>
-      </c>
-      <c r="G102" t="s">
-        <v>30</v>
-      </c>
-      <c r="I102" t="s">
-        <v>84</v>
-      </c>
-      <c r="J102" s="21">
-        <v>0.33600000000000002</v>
-      </c>
-    </row>
-    <row r="103" spans="1:13">
-      <c r="A103" t="s">
-        <v>2</v>
-      </c>
-      <c r="B103" t="s">
-        <v>7</v>
-      </c>
-      <c r="C103" t="s">
-        <v>38</v>
-      </c>
-      <c r="D103" t="s">
-        <v>27</v>
-      </c>
-      <c r="E103" t="s">
-        <v>15</v>
-      </c>
-      <c r="F103" t="s">
-        <v>29</v>
-      </c>
-      <c r="G103" t="s">
-        <v>30</v>
-      </c>
-      <c r="I103" t="s">
-        <v>84</v>
-      </c>
-      <c r="J103" s="21">
-        <v>0.44800000000000001</v>
-      </c>
-    </row>
-    <row r="104" spans="1:13">
-      <c r="A104" t="s">
-        <v>2</v>
-      </c>
-      <c r="B104" t="s">
-        <v>7</v>
-      </c>
-      <c r="C104" t="s">
-        <v>39</v>
-      </c>
-      <c r="D104" t="s">
-        <v>27</v>
-      </c>
-      <c r="E104" t="s">
-        <v>15</v>
-      </c>
-      <c r="F104" t="s">
-        <v>29</v>
-      </c>
-      <c r="G104" t="s">
-        <v>30</v>
-      </c>
-      <c r="I104" t="s">
-        <v>84</v>
-      </c>
-      <c r="J104" s="21">
-        <v>0.54600000000000004</v>
-      </c>
-    </row>
-    <row r="105" spans="1:13">
-      <c r="A105" t="s">
-        <v>2</v>
-      </c>
-      <c r="B105" t="s">
-        <v>7</v>
-      </c>
-      <c r="C105" t="s">
-        <v>40</v>
-      </c>
-      <c r="D105" t="s">
-        <v>27</v>
-      </c>
-      <c r="E105" t="s">
-        <v>15</v>
-      </c>
-      <c r="F105" t="s">
-        <v>29</v>
-      </c>
-      <c r="G105" t="s">
-        <v>30</v>
-      </c>
-      <c r="I105" t="s">
-        <v>84</v>
-      </c>
-      <c r="J105" s="21">
-        <v>0.63300000000000001</v>
-      </c>
-    </row>
-    <row r="106" spans="1:13">
-      <c r="A106" t="s">
-        <v>2</v>
-      </c>
-      <c r="B106" t="s">
-        <v>7</v>
-      </c>
-      <c r="C106" t="s">
-        <v>41</v>
-      </c>
-      <c r="D106" t="s">
-        <v>27</v>
-      </c>
-      <c r="E106" t="s">
-        <v>15</v>
-      </c>
-      <c r="F106" t="s">
-        <v>29</v>
-      </c>
-      <c r="G106" t="s">
-        <v>30</v>
-      </c>
-      <c r="I106" t="s">
-        <v>84</v>
-      </c>
-      <c r="J106" s="21">
+      <c r="J86" s="21">
         <v>0.67600000000000005</v>
       </c>
     </row>
+    <row r="91" spans="1:13" ht="15"/>
+    <row r="92" spans="1:13" ht="15"/>
+    <row r="97" ht="15"/>
+    <row r="102" ht="15"/>
   </sheetData>
   <dataValidations count="5">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:B1" xr:uid="{E441A666-11EF-40F7-A6AA-2528D8D84D13}"/>
@@ -6470,94 +5787,94 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="34" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="34"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
     </row>
     <row r="2" spans="1:17" ht="15">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33" t="s">
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33" t="s">
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33" t="s">
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="33"/>
-      <c r="P2" s="33"/>
-      <c r="Q2" s="33"/>
+      <c r="O2" s="34"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="34"/>
     </row>
     <row r="3" spans="1:17" ht="15">
       <c r="A3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33" t="s">
+      <c r="C3" s="34"/>
+      <c r="D3" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33" t="s">
+      <c r="E3" s="34"/>
+      <c r="F3" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33" t="s">
+      <c r="G3" s="34"/>
+      <c r="H3" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33" t="s">
+      <c r="I3" s="34"/>
+      <c r="J3" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33" t="s">
+      <c r="K3" s="34"/>
+      <c r="L3" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="M3" s="33"/>
-      <c r="N3" s="33" t="s">
+      <c r="M3" s="34"/>
+      <c r="N3" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33" t="s">
+      <c r="O3" s="34"/>
+      <c r="P3" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="Q3" s="33"/>
+      <c r="Q3" s="34"/>
     </row>
     <row r="4" spans="1:17" ht="15">
       <c r="A4" s="3" t="s">
@@ -7088,7 +6405,7 @@
         <v>47</v>
       </c>
       <c r="J8" s="7">
-        <v>0.61875637104994907</v>
+        <v>0.61875637104994896</v>
       </c>
       <c r="L8" s="9" t="s">
         <v>101</v>
@@ -7659,18 +6976,18 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="34" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="34"/>
+      <c r="F1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="34"/>
+      <c r="G1" s="35"/>
       <c r="H1" s="1" t="s">
         <v>26</v>
       </c>
@@ -9371,7 +8688,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="101.45">
+    <row r="2" spans="1:9" ht="115.5">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -9429,7 +8746,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" ht="57.75">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -9445,7 +8762,7 @@
       <c r="E4">
         <v>2012</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="5" t="s">
         <v>165</v>
       </c>
       <c r="G4">
@@ -9458,7 +8775,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" ht="43.5">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -9474,7 +8791,7 @@
       <c r="E5">
         <v>2013</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="5" t="s">
         <v>169</v>
       </c>
       <c r="G5">
@@ -9554,6 +8871,7 @@
     <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="150" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9680,7 +8998,7 @@
       <c r="H6" s="23"/>
       <c r="I6" s="23"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" ht="29.25">
       <c r="A7" s="26" t="s">
         <v>185</v>
       </c>
@@ -9692,7 +9010,7 @@
       <c r="E7" s="26" t="s">
         <v>189</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="33" t="s">
         <v>190</v>
       </c>
       <c r="G7" s="26"/>
@@ -9795,17 +9113,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100447C4EFE3BCDC24F9D43FB479AF7E97A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="710ccc9eba0c031f4d3c8297a7da4be2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19a3940c-c740-4699-845a-46837f99845a" xmlns:ns3="539a68f6-d0ac-4a73-9041-e1fa437c4cee" xmlns:ns4="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a67399e28ae6312d8947be2cafff42c1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="19a3940c-c740-4699-845a-46837f99845a"/>
@@ -10059,6 +9366,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ab06a5aa-8e31-4bdb-9b13-38c58a92ec8a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19a3940c-c740-4699-845a-46837f99845a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -10069,11 +9387,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302FEEF7-88D6-41D4-B999-EFF8511D95B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4173999B-2FEB-4E5B-A6C7-6E33DD5EA2F7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>